<commit_message>
2. Theories (75%) + 3. Methods
</commit_message>
<xml_diff>
--- a/meetings/AsymReca_ThkCalc.xlsx
+++ b/meetings/AsymReca_ThkCalc.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98DC32DB-07CD-4939-8228-6D731379F6A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="-120" windowWidth="28200" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="720" yWindow="-120" windowWidth="28200" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="532" sheetId="8" r:id="rId1"/>
@@ -2269,7 +2269,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2626,12 +2626,45 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2641,36 +2674,15 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2680,15 +2692,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -2698,20 +2710,35 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2731,37 +2758,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2770,24 +2767,14 @@
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="17">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2818,6 +2805,26 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2918,26 +2925,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3253,13 +3240,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="132" t="s">
+      <c r="C1" s="128" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
@@ -3268,50 +3255,50 @@
       <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="123" t="s">
+      <c r="G1" s="134" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="125" t="s">
+      <c r="H1" s="124" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="128" t="s">
+      <c r="J1" s="136" t="s">
         <v>28</v>
       </c>
       <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="131"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="138"/>
       <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="131"/>
+      <c r="O1" s="132"/>
+      <c r="P1" s="138"/>
       <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="127"/>
-      <c r="S1" s="131"/>
-      <c r="T1" s="120" t="s">
+      <c r="R1" s="132"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="126" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121"/>
+      <c r="A2" s="127"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="133"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="129"/>
+      <c r="C2" s="129"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="125"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="137"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -3339,11 +3326,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="121"/>
-      <c r="V2" s="122"/>
-      <c r="W2" s="122"/>
-      <c r="X2" s="122"/>
-      <c r="Y2" s="122"/>
+      <c r="T2" s="127"/>
+      <c r="V2" s="133"/>
+      <c r="W2" s="133"/>
+      <c r="X2" s="133"/>
+      <c r="Y2" s="133"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -4005,7 +3992,7 @@
         <v>6.0999999999999999E-2</v>
       </c>
       <c r="M14" s="97">
-        <f t="shared" ref="M14:M21" si="5">K14-L14</f>
+        <f t="shared" ref="M14:M18" si="5">K14-L14</f>
         <v>0.159</v>
       </c>
       <c r="N14" s="92">
@@ -4015,7 +4002,7 @@
         <v>0.84</v>
       </c>
       <c r="P14" s="97">
-        <f t="shared" ref="P14:P21" si="6">N14-O14</f>
+        <f t="shared" ref="P14:P18" si="6">N14-O14</f>
         <v>-5.9999999999999942E-2</v>
       </c>
       <c r="Q14" s="92">
@@ -4025,7 +4012,7 @@
         <v>0.1</v>
       </c>
       <c r="S14" s="97">
-        <f t="shared" ref="S14:S21" si="7">Q14-R14</f>
+        <f t="shared" ref="S14:S18" si="7">Q14-R14</f>
         <v>-0.1</v>
       </c>
     </row>
@@ -4270,13 +4257,13 @@
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A20" s="164" t="s">
+      <c r="A20" s="123" t="s">
         <v>94</v>
       </c>
-      <c r="C20" s="162" t="s">
+      <c r="C20" s="121" t="s">
         <v>95</v>
       </c>
-      <c r="E20" s="163" t="s">
+      <c r="E20" s="122" t="s">
         <v>89</v>
       </c>
       <c r="F20" s="34">
@@ -4331,11 +4318,11 @@
       <c r="A21" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="C21" s="165" t="s">
+      <c r="C21" s="32" t="s">
         <v>88</v>
       </c>
       <c r="D21" s="37"/>
-      <c r="E21" s="163" t="s">
+      <c r="E21" s="122" t="s">
         <v>89</v>
       </c>
       <c r="F21" s="34">
@@ -4348,7 +4335,7 @@
         <f>G21</f>
         <v>5.09</v>
       </c>
-      <c r="I21" s="161" t="s">
+      <c r="I21" s="120" t="s">
         <v>90</v>
       </c>
       <c r="J21" s="43">
@@ -4391,11 +4378,11 @@
         <v>92</v>
       </c>
       <c r="B22" s="32"/>
-      <c r="C22" s="165" t="s">
+      <c r="C22" s="32" t="s">
         <v>88</v>
       </c>
       <c r="D22" s="38"/>
-      <c r="E22" s="163" t="s">
+      <c r="E22" s="122" t="s">
         <v>89</v>
       </c>
       <c r="F22" s="34">
@@ -4408,7 +4395,7 @@
         <f>G22</f>
         <v>7.6</v>
       </c>
-      <c r="I22" s="161" t="s">
+      <c r="I22" s="120" t="s">
         <v>93</v>
       </c>
       <c r="J22" s="43">
@@ -4611,11 +4598,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
@@ -4625,23 +4607,28 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:P1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="Q1:S1"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M18">
-    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="greaterThan">
       <formula>$M$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M40:M42">
-    <cfRule type="cellIs" dxfId="16" priority="4" operator="greaterThan">
-      <formula>0.45</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="greaterThan">
-      <formula>0.45</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M20:M21">
     <cfRule type="cellIs" dxfId="15" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M40:M42">
+    <cfRule type="cellIs" dxfId="14" priority="4" operator="greaterThan">
+      <formula>0.45</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="greaterThan">
+      <formula>0.45</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -4679,13 +4666,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="136" t="s">
+      <c r="C1" s="140" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
@@ -4694,50 +4681,50 @@
       <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="123" t="s">
+      <c r="G1" s="134" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="135" t="s">
+      <c r="H1" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="128" t="s">
+      <c r="J1" s="136" t="s">
         <v>28</v>
       </c>
       <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="131"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="138"/>
       <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="131"/>
+      <c r="O1" s="132"/>
+      <c r="P1" s="138"/>
       <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="127"/>
-      <c r="S1" s="131"/>
-      <c r="T1" s="120" t="s">
+      <c r="R1" s="132"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="126" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121"/>
+      <c r="A2" s="127"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="137"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="121"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="129"/>
+      <c r="C2" s="141"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="137"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -4765,11 +4752,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="121"/>
-      <c r="V2" s="122"/>
-      <c r="W2" s="122"/>
-      <c r="X2" s="122"/>
-      <c r="Y2" s="122"/>
+      <c r="T2" s="127"/>
+      <c r="V2" s="133"/>
+      <c r="W2" s="133"/>
+      <c r="X2" s="133"/>
+      <c r="Y2" s="133"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -5692,12 +5679,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -5706,15 +5687,21 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M4:M17">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -5753,13 +5740,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="136" t="s">
+      <c r="C1" s="140" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
@@ -5768,50 +5755,50 @@
       <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="123" t="s">
+      <c r="G1" s="134" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="135" t="s">
+      <c r="H1" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="128" t="s">
+      <c r="J1" s="136" t="s">
         <v>28</v>
       </c>
       <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="131"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="138"/>
       <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="131"/>
+      <c r="O1" s="132"/>
+      <c r="P1" s="138"/>
       <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="127"/>
-      <c r="S1" s="131"/>
-      <c r="T1" s="120" t="s">
+      <c r="R1" s="132"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="126" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121"/>
+      <c r="A2" s="127"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="137"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="121"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="129"/>
+      <c r="C2" s="141"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="137"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -5839,11 +5826,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="121"/>
-      <c r="V2" s="122"/>
-      <c r="W2" s="122"/>
-      <c r="X2" s="122"/>
-      <c r="Y2" s="122"/>
+      <c r="T2" s="127"/>
+      <c r="V2" s="133"/>
+      <c r="W2" s="133"/>
+      <c r="X2" s="133"/>
+      <c r="Y2" s="133"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -6507,12 +6494,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -6521,14 +6502,20 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M12">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -6567,13 +6554,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="136" t="s">
+      <c r="C1" s="140" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
@@ -6582,50 +6569,50 @@
       <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="123" t="s">
+      <c r="G1" s="134" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="135" t="s">
+      <c r="H1" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="128" t="s">
+      <c r="J1" s="136" t="s">
         <v>28</v>
       </c>
       <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="131"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="138"/>
       <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="131"/>
+      <c r="O1" s="132"/>
+      <c r="P1" s="138"/>
       <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="127"/>
-      <c r="S1" s="131"/>
-      <c r="T1" s="120" t="s">
+      <c r="R1" s="132"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="126" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121"/>
+      <c r="A2" s="127"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="137"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="121"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="129"/>
+      <c r="C2" s="141"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="137"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -6653,11 +6640,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="121"/>
-      <c r="V2" s="122"/>
-      <c r="W2" s="122"/>
-      <c r="X2" s="122"/>
-      <c r="Y2" s="122"/>
+      <c r="T2" s="127"/>
+      <c r="V2" s="133"/>
+      <c r="W2" s="133"/>
+      <c r="X2" s="133"/>
+      <c r="Y2" s="133"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -7200,6 +7187,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -7208,20 +7201,14 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M7 M10:M11">
-    <cfRule type="cellIs" dxfId="10" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -7260,13 +7247,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="132" t="s">
+      <c r="C1" s="128" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
@@ -7275,50 +7262,50 @@
       <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="123" t="s">
+      <c r="G1" s="134" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="125" t="s">
+      <c r="H1" s="124" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="128" t="s">
+      <c r="J1" s="136" t="s">
         <v>28</v>
       </c>
       <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="131"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="138"/>
       <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="131"/>
+      <c r="O1" s="132"/>
+      <c r="P1" s="138"/>
       <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="127"/>
-      <c r="S1" s="131"/>
-      <c r="T1" s="120" t="s">
+      <c r="R1" s="132"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="126" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121"/>
+      <c r="A2" s="127"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="133"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="129"/>
+      <c r="C2" s="129"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="125"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="137"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -7346,11 +7333,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="121"/>
-      <c r="V2" s="122"/>
-      <c r="W2" s="122"/>
-      <c r="X2" s="122"/>
-      <c r="Y2" s="122"/>
+      <c r="T2" s="127"/>
+      <c r="V2" s="133"/>
+      <c r="W2" s="133"/>
+      <c r="X2" s="133"/>
+      <c r="Y2" s="133"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -8424,7 +8411,7 @@
       <c r="C24" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="E24" s="163" t="s">
+      <c r="E24" s="122" t="s">
         <v>99</v>
       </c>
       <c r="F24" s="34">
@@ -8478,19 +8465,19 @@
       <c r="A25" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="C25" s="165" t="s">
+      <c r="C25" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="E25" s="163"/>
+      <c r="E25" s="122"/>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="C26" s="165" t="s">
+      <c r="C26" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="E26" s="163"/>
+      <c r="E26" s="122"/>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="30"/>
@@ -8525,12 +8512,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -8539,14 +8520,20 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M17 M19">
-    <cfRule type="cellIs" dxfId="8" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="4" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M16:M18">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="6" operator="greaterThan">
@@ -8554,12 +8541,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M20:M22">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
       <formula>$M$19</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M24">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8595,66 +8582,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="142" t="s">
+      <c r="A1" s="146" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="120" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="143" t="s">
+      <c r="B1" s="126" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="147" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="132" t="s">
+      <c r="D1" s="128" t="s">
         <v>11</v>
       </c>
       <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="135" t="s">
+      <c r="G1" s="139" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="135" t="s">
+      <c r="H1" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="128" t="s">
+      <c r="J1" s="136" t="s">
         <v>28</v>
       </c>
       <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="131"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="138"/>
       <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="131"/>
+      <c r="O1" s="132"/>
+      <c r="P1" s="138"/>
       <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="127"/>
-      <c r="S1" s="131"/>
-      <c r="T1" s="142" t="s">
+      <c r="R1" s="132"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="146" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="122"/>
-      <c r="B2" s="121"/>
-      <c r="C2" s="137"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="121"/>
-      <c r="H2" s="121"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="129"/>
+      <c r="A2" s="133"/>
+      <c r="B2" s="127"/>
+      <c r="C2" s="141"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="137"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -8682,11 +8669,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="122"/>
-      <c r="V2" s="122"/>
-      <c r="W2" s="122"/>
-      <c r="X2" s="122"/>
-      <c r="Y2" s="122"/>
+      <c r="T2" s="133"/>
+      <c r="V2" s="133"/>
+      <c r="W2" s="133"/>
+      <c r="X2" s="133"/>
+      <c r="Y2" s="133"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="46">
@@ -8756,16 +8743,16 @@
       <c r="D4" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="138">
+      <c r="E4" s="143">
         <v>32.700000000000003</v>
       </c>
-      <c r="F4" s="139">
+      <c r="F4" s="144">
         <v>90.1</v>
       </c>
-      <c r="G4" s="141">
+      <c r="G4" s="145">
         <v>38.5</v>
       </c>
-      <c r="H4" s="141"/>
+      <c r="H4" s="145"/>
       <c r="I4" s="66">
         <v>18.3</v>
       </c>
@@ -8808,12 +8795,12 @@
       <c r="D5" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="138"/>
-      <c r="F5" s="139"/>
-      <c r="G5" s="140">
+      <c r="E5" s="143"/>
+      <c r="F5" s="144"/>
+      <c r="G5" s="142">
         <v>41.2</v>
       </c>
-      <c r="H5" s="140"/>
+      <c r="H5" s="142"/>
       <c r="I5" s="58">
         <v>15.1</v>
       </c>
@@ -8858,12 +8845,12 @@
       <c r="D6" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="138"/>
-      <c r="F6" s="139"/>
-      <c r="G6" s="140">
+      <c r="E6" s="143"/>
+      <c r="F6" s="144"/>
+      <c r="G6" s="142">
         <v>24.3</v>
       </c>
-      <c r="H6" s="140"/>
+      <c r="H6" s="142"/>
       <c r="I6" s="58">
         <v>30.6</v>
       </c>
@@ -8905,12 +8892,12 @@
       <c r="D7" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="138"/>
-      <c r="F7" s="139"/>
-      <c r="G7" s="140">
+      <c r="E7" s="143"/>
+      <c r="F7" s="144"/>
+      <c r="G7" s="142">
         <v>42.6</v>
       </c>
-      <c r="H7" s="140"/>
+      <c r="H7" s="142"/>
       <c r="I7" s="58">
         <v>13.3</v>
       </c>
@@ -8954,12 +8941,12 @@
       <c r="D8" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="138"/>
-      <c r="F8" s="139"/>
-      <c r="G8" s="140">
+      <c r="E8" s="143"/>
+      <c r="F8" s="144"/>
+      <c r="G8" s="142">
         <v>31.9</v>
       </c>
-      <c r="H8" s="140"/>
+      <c r="H8" s="142"/>
       <c r="I8" s="58">
         <v>23.7</v>
       </c>
@@ -9001,8 +8988,8 @@
       <c r="D9" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="138"/>
-      <c r="F9" s="139"/>
+      <c r="E9" s="143"/>
+      <c r="F9" s="144"/>
       <c r="G9" s="66">
         <v>2.7</v>
       </c>
@@ -9051,8 +9038,8 @@
       <c r="D10" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="138"/>
-      <c r="F10" s="139"/>
+      <c r="E10" s="143"/>
+      <c r="F10" s="144"/>
       <c r="G10" s="58">
         <v>4.2</v>
       </c>
@@ -9101,8 +9088,8 @@
       <c r="D11" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="138"/>
-      <c r="F11" s="139"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="144"/>
       <c r="G11" s="58">
         <v>1.3</v>
       </c>
@@ -9220,16 +9207,16 @@
       <c r="D14" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="138">
+      <c r="E14" s="143">
         <v>66.599999999999994</v>
       </c>
-      <c r="F14" s="139">
+      <c r="F14" s="144">
         <v>181.3</v>
       </c>
-      <c r="G14" s="140">
+      <c r="G14" s="142">
         <v>107.3</v>
       </c>
-      <c r="H14" s="140"/>
+      <c r="H14" s="142"/>
       <c r="I14" s="58">
         <v>0</v>
       </c>
@@ -9271,12 +9258,12 @@
       <c r="D15" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="138"/>
-      <c r="F15" s="139"/>
-      <c r="G15" s="141">
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
+      <c r="G15" s="145">
         <v>68.7</v>
       </c>
-      <c r="H15" s="141"/>
+      <c r="H15" s="145"/>
       <c r="I15" s="66">
         <v>51.9</v>
       </c>
@@ -9319,12 +9306,12 @@
       <c r="D16" s="81" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="138"/>
-      <c r="F16" s="139"/>
-      <c r="G16" s="141">
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="145">
         <v>105</v>
       </c>
-      <c r="H16" s="141"/>
+      <c r="H16" s="145"/>
       <c r="I16" s="66">
         <v>0</v>
       </c>
@@ -9367,12 +9354,12 @@
       <c r="D17" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="138"/>
-      <c r="F17" s="139"/>
-      <c r="G17" s="140">
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
+      <c r="G17" s="142">
         <v>65.599999999999994</v>
       </c>
-      <c r="H17" s="140"/>
+      <c r="H17" s="142"/>
       <c r="I17" s="58">
         <v>53.5</v>
       </c>
@@ -9415,8 +9402,8 @@
       <c r="D18" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="138"/>
-      <c r="F18" s="139"/>
+      <c r="E18" s="143"/>
+      <c r="F18" s="144"/>
       <c r="G18" s="58">
         <v>42.6</v>
       </c>
@@ -9465,8 +9452,8 @@
       <c r="D19" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="138"/>
-      <c r="F19" s="139"/>
+      <c r="E19" s="143"/>
+      <c r="F19" s="144"/>
       <c r="G19" s="58">
         <v>47.7</v>
       </c>
@@ -9515,8 +9502,8 @@
       <c r="D20" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="138"/>
-      <c r="F20" s="139"/>
+      <c r="E20" s="143"/>
+      <c r="F20" s="144"/>
       <c r="G20" s="58">
         <v>48.7</v>
       </c>
@@ -9672,18 +9659,12 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="E4:E11"/>
-    <mergeCell ref="F4:F11"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="E14:E20"/>
+    <mergeCell ref="F14:F20"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G14:H14"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
@@ -9695,20 +9676,26 @@
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
-    <mergeCell ref="E14:E20"/>
-    <mergeCell ref="F14:F20"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="E4:E11"/>
+    <mergeCell ref="F4:F11"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
   </mergeCells>
   <conditionalFormatting sqref="M14:M20">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
       <formula>$M$13</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M29:M33">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -9747,66 +9734,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="142" t="s">
+      <c r="A1" s="146" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="120" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="143" t="s">
+      <c r="B1" s="126" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="147" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="132" t="s">
+      <c r="D1" s="128" t="s">
         <v>11</v>
       </c>
       <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="135" t="s">
+      <c r="G1" s="139" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="135" t="s">
+      <c r="H1" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="128" t="s">
+      <c r="J1" s="136" t="s">
         <v>28</v>
       </c>
       <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="127"/>
-      <c r="M1" s="131"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="138"/>
       <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="131"/>
+      <c r="O1" s="132"/>
+      <c r="P1" s="138"/>
       <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="127"/>
-      <c r="S1" s="131"/>
-      <c r="T1" s="144" t="s">
+      <c r="R1" s="132"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="151" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="122"/>
-      <c r="B2" s="121"/>
-      <c r="C2" s="137"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="121"/>
-      <c r="H2" s="121"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="129"/>
+      <c r="A2" s="133"/>
+      <c r="B2" s="127"/>
+      <c r="C2" s="141"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="137"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -9834,11 +9821,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="145"/>
-      <c r="V2" s="122"/>
-      <c r="W2" s="122"/>
-      <c r="X2" s="122"/>
-      <c r="Y2" s="122"/>
+      <c r="T2" s="152"/>
+      <c r="V2" s="133"/>
+      <c r="W2" s="133"/>
+      <c r="X2" s="133"/>
+      <c r="Y2" s="133"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="30">
@@ -9850,10 +9837,10 @@
       <c r="D3" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="146">
-        <v>0</v>
-      </c>
-      <c r="F3" s="148">
+      <c r="E3" s="148">
+        <v>0</v>
+      </c>
+      <c r="F3" s="150">
         <v>0</v>
       </c>
       <c r="G3" s="58">
@@ -9905,8 +9892,8 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E4" s="147"/>
-      <c r="F4" s="140"/>
+      <c r="E4" s="149"/>
+      <c r="F4" s="142"/>
       <c r="G4" s="58">
         <v>35.6</v>
       </c>
@@ -9959,10 +9946,10 @@
       <c r="D5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="138">
+      <c r="E5" s="143">
         <v>32.700000000000003</v>
       </c>
-      <c r="F5" s="139">
+      <c r="F5" s="144">
         <v>90.1</v>
       </c>
       <c r="G5" s="58">
@@ -10015,8 +10002,8 @@
       <c r="D6" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="138"/>
-      <c r="F6" s="139"/>
+      <c r="E6" s="143"/>
+      <c r="F6" s="144"/>
       <c r="G6" s="58">
         <v>35.6</v>
       </c>
@@ -10139,10 +10126,10 @@
       <c r="D9" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="138">
+      <c r="E9" s="143">
         <v>66.599999999999994</v>
       </c>
-      <c r="F9" s="139">
+      <c r="F9" s="144">
         <v>181.3</v>
       </c>
       <c r="G9" s="58">
@@ -10194,8 +10181,8 @@
       <c r="D10" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="138"/>
-      <c r="F10" s="139"/>
+      <c r="E10" s="143"/>
+      <c r="F10" s="144"/>
       <c r="G10" s="58">
         <v>75.8</v>
       </c>
@@ -10245,8 +10232,8 @@
       <c r="D11" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="138"/>
-      <c r="F11" s="139"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="144"/>
       <c r="G11" s="58">
         <v>89.5</v>
       </c>
@@ -10294,8 +10281,8 @@
       <c r="D12" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="138"/>
-      <c r="F12" s="139"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="144"/>
       <c r="G12" s="58">
         <v>46.1</v>
       </c>
@@ -10345,8 +10332,8 @@
       <c r="D13" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="138"/>
-      <c r="F13" s="139"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="58">
         <v>73.400000000000006</v>
       </c>
@@ -10395,8 +10382,8 @@
       <c r="D14" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="138"/>
-      <c r="F14" s="139"/>
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
       <c r="G14" s="58">
         <v>88.4</v>
       </c>
@@ -10445,8 +10432,8 @@
       <c r="D15" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="138"/>
-      <c r="F15" s="139"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="58">
         <v>27.5</v>
       </c>
@@ -10495,8 +10482,8 @@
       <c r="D16" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="138"/>
-      <c r="F16" s="139"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
       <c r="G16" s="58">
         <v>94.8</v>
       </c>
@@ -10545,8 +10532,8 @@
       <c r="D17" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="138"/>
-      <c r="F17" s="139"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
       <c r="G17" s="58">
         <v>861.6</v>
       </c>
@@ -10598,8 +10585,8 @@
       <c r="D18" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="138"/>
-      <c r="F18" s="139"/>
+      <c r="E18" s="143"/>
+      <c r="F18" s="144"/>
       <c r="G18" s="58">
         <v>48.1</v>
       </c>
@@ -10648,8 +10635,8 @@
       <c r="D19" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="138"/>
-      <c r="F19" s="139"/>
+      <c r="E19" s="143"/>
+      <c r="F19" s="144"/>
       <c r="G19" s="58">
         <v>41.8</v>
       </c>
@@ -10704,6 +10691,14 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
     <mergeCell ref="E9:E19"/>
     <mergeCell ref="F9:F19"/>
     <mergeCell ref="B1:B2"/>
@@ -10718,18 +10713,10 @@
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:P1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M9:M19">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -10737,7 +10724,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M9:M20">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>$M$8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10759,40 +10746,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="156" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="160" t="s">
+      <c r="B1" s="156" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="155" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="155" t="s">
+      <c r="C1" s="157" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="157" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="155" t="s">
+      <c r="E1" s="157" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="156" t="s">
+      <c r="F1" s="164" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="156"/>
-      <c r="H1" s="149" t="s">
+      <c r="G1" s="164"/>
+      <c r="H1" s="158" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="149"/>
-      <c r="J1" s="150" t="s">
+      <c r="I1" s="158"/>
+      <c r="J1" s="159" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="150"/>
+      <c r="K1" s="159"/>
     </row>
     <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="160"/>
-      <c r="B2" s="160"/>
-      <c r="C2" s="155"/>
-      <c r="D2" s="155"/>
-      <c r="E2" s="155"/>
+      <c r="A2" s="156"/>
+      <c r="B2" s="156"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
       <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
@@ -10813,16 +10800,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="151" t="s">
+      <c r="A3" s="160" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="151">
+      <c r="C3" s="160">
         <v>1550</v>
       </c>
-      <c r="D3" s="151" t="s">
+      <c r="D3" s="160" t="s">
         <v>26</v>
       </c>
       <c r="E3" s="13">
@@ -10848,12 +10835,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="152"/>
+      <c r="A4" s="161"/>
       <c r="B4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="152"/>
-      <c r="D4" s="154"/>
+      <c r="C4" s="161"/>
+      <c r="D4" s="163"/>
       <c r="E4" s="18">
         <v>52</v>
       </c>
@@ -10877,11 +10864,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="152"/>
+      <c r="A5" s="161"/>
       <c r="B5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="152"/>
+      <c r="C5" s="161"/>
       <c r="D5" s="19" t="s">
         <v>14</v>
       </c>
@@ -10909,11 +10896,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="153"/>
+      <c r="A6" s="162"/>
       <c r="B6" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="153"/>
+      <c r="C6" s="162"/>
       <c r="D6" s="23" t="s">
         <v>15</v>
       </c>
@@ -10941,16 +10928,16 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="157" t="s">
+      <c r="A7" s="153" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="157">
+      <c r="C7" s="153">
         <v>1320</v>
       </c>
-      <c r="D7" s="157" t="s">
+      <c r="D7" s="153" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="3">
@@ -10976,12 +10963,12 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="158"/>
+      <c r="A8" s="154"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="158"/>
-      <c r="D8" s="159"/>
+      <c r="C8" s="154"/>
+      <c r="D8" s="155"/>
       <c r="E8" s="1">
         <v>100</v>
       </c>
@@ -11005,11 +10992,11 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="158"/>
+      <c r="A9" s="154"/>
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="158"/>
+      <c r="C9" s="154"/>
       <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
@@ -11037,11 +11024,11 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="158"/>
+      <c r="A10" s="154"/>
       <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="158"/>
+      <c r="C10" s="154"/>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
@@ -11069,11 +11056,11 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="159"/>
+      <c r="A11" s="155"/>
       <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="159"/>
+      <c r="C11" s="155"/>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
@@ -11102,6 +11089,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:G1"/>
     <mergeCell ref="A7:A11"/>
     <mergeCell ref="C7:C11"/>
     <mergeCell ref="D7:D8"/>
@@ -11109,13 +11103,6 @@
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11134,40 +11121,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="156" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="160" t="s">
+      <c r="B1" s="156" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="155" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="155" t="s">
+      <c r="C1" s="157" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="157" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="155" t="s">
+      <c r="E1" s="157" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="156" t="s">
+      <c r="F1" s="164" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="156"/>
-      <c r="H1" s="149" t="s">
+      <c r="G1" s="164"/>
+      <c r="H1" s="158" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="149"/>
-      <c r="J1" s="150" t="s">
+      <c r="I1" s="158"/>
+      <c r="J1" s="159" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="150"/>
+      <c r="K1" s="159"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="160"/>
-      <c r="B2" s="160"/>
-      <c r="C2" s="155"/>
-      <c r="D2" s="155"/>
-      <c r="E2" s="155"/>
+      <c r="A2" s="156"/>
+      <c r="B2" s="156"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
       <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
@@ -11188,16 +11175,16 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="157" t="s">
+      <c r="A3" s="153" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="157">
+      <c r="C3" s="153">
         <v>1320</v>
       </c>
-      <c r="D3" s="157" t="s">
+      <c r="D3" s="153" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="3">
@@ -11223,12 +11210,12 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="158"/>
+      <c r="A4" s="154"/>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="158"/>
-      <c r="D4" s="159"/>
+      <c r="C4" s="154"/>
+      <c r="D4" s="155"/>
       <c r="E4" s="1">
         <v>100</v>
       </c>
@@ -11252,11 +11239,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="158"/>
+      <c r="A5" s="154"/>
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="158"/>
+      <c r="C5" s="154"/>
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
@@ -11284,11 +11271,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="158"/>
+      <c r="A6" s="154"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="158"/>
+      <c r="C6" s="154"/>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
@@ -11316,11 +11303,11 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="159"/>
+      <c r="A7" s="155"/>
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="159"/>
+      <c r="C7" s="155"/>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
Before change to OptCommun
</commit_message>
<xml_diff>
--- a/meetings/AsymReca_ThkCalc.xlsx
+++ b/meetings/AsymReca_ThkCalc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2024-ILLUSTRIOUS\My Drive (61050734@kmitl.ac.th)\AsymReca_SbSe\meetings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98DC32DB-07CD-4939-8228-6D731379F6A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2930F64-1CFB-415C-91FC-D7054F5D9ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="-120" windowWidth="28200" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="532" sheetId="8" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="800" sheetId="12" r:id="rId4"/>
     <sheet name="1064" sheetId="9" r:id="rId5"/>
     <sheet name="Amorphous phase" sheetId="7" state="hidden" r:id="rId6"/>
-    <sheet name="Crystalline phase" sheetId="4" r:id="rId7"/>
+    <sheet name="Crystalline" sheetId="4" r:id="rId7"/>
     <sheet name="Sheet2" sheetId="5" state="hidden" r:id="rId8"/>
     <sheet name="Sheet3" sheetId="6" state="hidden" r:id="rId9"/>
   </sheets>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="98">
   <si>
     <t>Wavelength (nm)</t>
   </si>
@@ -1830,15 +1830,6 @@
     <t>Peak absorption</t>
   </si>
   <si>
-    <t>500-680</t>
-  </si>
-  <si>
-    <t>520-610</t>
-  </si>
-  <si>
-    <t>530-580</t>
-  </si>
-  <si>
     <t>520-630</t>
   </si>
   <si>
@@ -1909,6 +1900,9 @@
   </si>
   <si>
     <t>tH=133.23</t>
+  </si>
+  <si>
+    <t>MaxT shifted to 1302</t>
   </si>
 </sst>
 </file>
@@ -2269,7 +2263,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2760,6 +2754,18 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3340,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D3" s="37">
         <v>0</v>
@@ -3402,7 +3408,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D4" s="38">
         <v>0</v>
@@ -3463,7 +3469,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D5" s="38">
         <v>0</v>
@@ -3524,7 +3530,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="81" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D6" s="38">
         <v>0</v>
@@ -3586,7 +3592,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D7" s="38">
         <v>1</v>
@@ -3647,7 +3653,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D8" s="38">
         <v>2</v>
@@ -3708,7 +3714,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D9" s="38">
         <v>2</v>
@@ -3769,7 +3775,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D10" s="38">
         <v>3</v>
@@ -3829,7 +3835,7 @@
         <v>2</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D11" s="38">
         <v>3</v>
@@ -3900,7 +3906,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="81" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D13" s="38">
         <v>1</v>
@@ -3961,7 +3967,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D14" s="38">
         <v>2</v>
@@ -4021,7 +4027,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="81" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D15" s="38">
         <v>2</v>
@@ -4081,7 +4087,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D16" s="38">
         <v>3</v>
@@ -4141,7 +4147,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D17" s="38">
         <v>3</v>
@@ -4201,7 +4207,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D18" s="38">
         <v>3</v>
@@ -4258,13 +4264,13 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="123" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C20" s="121" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E20" s="122" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F20" s="34">
         <v>96.08</v>
@@ -4316,14 +4322,14 @@
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="30" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C21" s="32" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D21" s="37"/>
       <c r="E21" s="122" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F21" s="34">
         <v>96.08</v>
@@ -4336,7 +4342,7 @@
         <v>5.09</v>
       </c>
       <c r="I21" s="120" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="J21" s="43">
         <v>218.5</v>
@@ -4375,15 +4381,15 @@
     </row>
     <row r="22" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B22" s="32"/>
       <c r="C22" s="32" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D22" s="38"/>
       <c r="E22" s="122" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F22" s="34">
         <v>96.08</v>
@@ -4396,7 +4402,7 @@
         <v>7.6</v>
       </c>
       <c r="I22" s="120" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="J22" s="43">
         <f>217.7</f>
@@ -4442,10 +4448,10 @@
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="30"/>
       <c r="B24" s="30" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="M24" s="109"/>
       <c r="P24" s="97"/>
@@ -4454,7 +4460,7 @@
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="30" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B25" s="32">
         <v>3.9615</v>
@@ -4470,7 +4476,7 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="30" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B26" s="108">
         <v>4.7876000000000003</v>
@@ -4766,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D3" s="38">
         <v>0</v>
@@ -4827,7 +4833,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D4" s="38">
         <v>0</v>
@@ -4888,7 +4894,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D5" s="38">
         <v>1</v>
@@ -4949,7 +4955,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D6" s="32">
         <v>1</v>
@@ -5009,7 +5015,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D7" s="38">
         <v>2</v>
@@ -5069,7 +5075,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D8" s="38">
         <v>2</v>
@@ -5130,7 +5136,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="108" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D9" s="38">
         <v>2</v>
@@ -5191,7 +5197,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="108" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D10" s="38">
         <v>3</v>
@@ -5253,7 +5259,7 @@
         <v>2</v>
       </c>
       <c r="C11" s="108" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D11" s="117">
         <v>3</v>
@@ -5318,7 +5324,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D13" s="38">
         <v>1</v>
@@ -5378,7 +5384,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D14" s="38">
         <v>2</v>
@@ -5438,7 +5444,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="38" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D15" s="38">
         <v>2</v>
@@ -5497,7 +5503,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D16" s="38">
         <v>3</v>
@@ -5557,7 +5563,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D17" s="38">
         <v>3</v>
@@ -5628,10 +5634,10 @@
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="30"/>
       <c r="B20" s="30" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H20" s="98"/>
       <c r="M20" s="97"/>
@@ -5640,7 +5646,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="30" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" s="32">
         <v>4.0286999999999997</v>
@@ -5656,7 +5662,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="30" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B22" s="108">
         <v>5.0734000000000004</v>
@@ -5840,7 +5846,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D3" s="38">
         <v>0</v>
@@ -5901,7 +5907,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D4" s="38">
         <v>0</v>
@@ -5962,7 +5968,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D5" s="38">
         <v>0</v>
@@ -6023,7 +6029,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D6" s="32">
         <v>1</v>
@@ -6083,7 +6089,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D7" s="38">
         <v>2</v>
@@ -6143,7 +6149,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D8" s="38">
         <v>1</v>
@@ -6204,7 +6210,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D9" s="38">
         <v>2</v>
@@ -6276,7 +6282,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D11" s="38">
         <v>2</v>
@@ -6337,7 +6343,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D12" s="38">
         <v>3</v>
@@ -6442,10 +6448,10 @@
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="30"/>
       <c r="B20" s="30" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H20" s="98"/>
       <c r="M20" s="97"/>
@@ -6454,7 +6460,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="30" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" s="32">
         <v>3.9072</v>
@@ -6470,7 +6476,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="30" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B22" s="108">
         <v>5.1289999999999996</v>
@@ -6654,7 +6660,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D3" s="38">
         <v>0</v>
@@ -6716,7 +6722,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D4" s="38">
         <v>0</v>
@@ -6777,7 +6783,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D5" s="38">
         <v>1</v>
@@ -6838,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D6" s="32">
         <v>1</v>
@@ -6898,7 +6904,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="108" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D7" s="38">
         <v>2</v>
@@ -6964,7 +6970,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D10" s="38">
         <v>1</v>
@@ -7026,7 +7032,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D11" s="38">
         <v>2</v>
@@ -7135,10 +7141,10 @@
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="30"/>
       <c r="B20" s="30" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H20" s="98"/>
       <c r="M20" s="97"/>
@@ -7147,7 +7153,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="30" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" s="32">
         <v>3.6627000000000001</v>
@@ -7163,7 +7169,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="30" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B22" s="108">
         <v>4.9420000000000002</v>
@@ -7221,7 +7227,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C373C9F4-FBF0-43BC-93B8-9C26388C4D3B}">
-  <dimension ref="A1:Y29"/>
+  <dimension ref="A1:Y30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" style="32" bestFit="1" customWidth="1"/>
@@ -7241,7 +7247,7 @@
     <col min="16" max="16" width="7.28515625" style="41" customWidth="1"/>
     <col min="17" max="18" width="7.28515625" style="92" customWidth="1"/>
     <col min="19" max="19" width="7.28515625" style="41" customWidth="1"/>
-    <col min="20" max="20" width="12.5703125" style="32" customWidth="1"/>
+    <col min="20" max="20" width="12.5703125" style="35" customWidth="1"/>
     <col min="21" max="25" width="7.28515625" style="32" customWidth="1"/>
     <col min="26" max="16384" width="9.140625" style="32"/>
   </cols>
@@ -7292,8 +7298,8 @@
       </c>
       <c r="R1" s="132"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="126" t="s">
-        <v>72</v>
+      <c r="T1" s="166" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -7333,7 +7339,7 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="127"/>
+      <c r="T2" s="167"/>
       <c r="V2" s="133"/>
       <c r="W2" s="133"/>
       <c r="X2" s="133"/>
@@ -7347,7 +7353,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D3" s="30">
         <v>0</v>
@@ -7376,11 +7382,11 @@
         <v>1</v>
       </c>
       <c r="L3" s="96">
-        <v>0.28599999999999998</v>
+        <v>0.28699999999999998</v>
       </c>
       <c r="M3" s="90">
         <f t="shared" ref="M3:M6" si="0">K3-L3</f>
-        <v>0.71399999999999997</v>
+        <v>0.71300000000000008</v>
       </c>
       <c r="N3" s="96">
         <v>3.3299999999999999E-16</v>
@@ -7396,14 +7402,14 @@
         <v>0</v>
       </c>
       <c r="R3" s="96">
-        <v>0.70099999999999996</v>
+        <v>0.7</v>
       </c>
       <c r="S3" s="90">
         <f t="shared" ref="S3:S6" si="2">Q3-R3</f>
-        <v>-0.70099999999999996</v>
-      </c>
-      <c r="T3" s="30" t="s">
-        <v>73</v>
+        <v>-0.7</v>
+      </c>
+      <c r="T3" s="35" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
@@ -7411,7 +7417,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="81" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D4" s="38">
         <v>1</v>
@@ -7465,16 +7471,13 @@
         <f t="shared" si="2"/>
         <v>-0.44</v>
       </c>
-      <c r="T4" s="32" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B5" s="32">
         <v>2</v>
       </c>
       <c r="C5" s="81" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D5" s="38">
         <v>2</v>
@@ -7528,16 +7531,14 @@
         <f t="shared" si="2"/>
         <v>-0.72199999999999998</v>
       </c>
-      <c r="T5" s="34" t="s">
-        <v>75</v>
-      </c>
+      <c r="T5" s="71"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B6" s="32">
         <v>3</v>
       </c>
       <c r="C6" s="81" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D6" s="38">
         <v>3</v>
@@ -7591,7 +7592,7 @@
         <f t="shared" si="2"/>
         <v>-0.89600000000000002</v>
       </c>
-      <c r="T6" s="34"/>
+      <c r="T6" s="71"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C7" s="38"/>
@@ -8148,10 +8149,7 @@
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="H18" s="98">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="H18" s="98"/>
       <c r="K18" s="92"/>
     </row>
     <row r="19" spans="1:20" s="101" customFormat="1" x14ac:dyDescent="0.25">
@@ -8160,7 +8158,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="119" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D19" s="101">
         <v>0</v>
@@ -8214,7 +8212,7 @@
         <f>R19-Q19</f>
         <v>-0.48499999999999999</v>
       </c>
-      <c r="T19" s="87">
+      <c r="T19" s="168">
         <v>597</v>
       </c>
     </row>
@@ -8223,7 +8221,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="119" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D20" s="38">
         <v>1</v>
@@ -8277,8 +8275,8 @@
         <f>R20-Q20</f>
         <v>-0.26500000000000001</v>
       </c>
-      <c r="T20" s="34" t="s">
-        <v>76</v>
+      <c r="T20" s="71" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
@@ -8286,7 +8284,7 @@
         <v>2</v>
       </c>
       <c r="C21" s="119" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D21" s="38">
         <v>2</v>
@@ -8340,8 +8338,8 @@
         <f>R21-Q21</f>
         <v>-0.55600000000000005</v>
       </c>
-      <c r="T21" s="34" t="s">
-        <v>76</v>
+      <c r="T21" s="71" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
@@ -8349,7 +8347,7 @@
         <v>3</v>
       </c>
       <c r="C22" s="119" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D22" s="38">
         <v>3</v>
@@ -8404,109 +8402,126 @@
         <v>-0.81100000000000005</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C23" s="165"/>
+      <c r="M23" s="97"/>
+      <c r="P23" s="97"/>
+      <c r="S23" s="97"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="32">
+        <v>0</v>
+      </c>
+      <c r="D24" s="38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="46" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="122" t="s">
         <v>96</v>
       </c>
-      <c r="C24" s="46" t="s">
-        <v>97</v>
-      </c>
-      <c r="E24" s="122" t="s">
-        <v>99</v>
-      </c>
-      <c r="F24" s="34">
+      <c r="F25" s="34">
         <v>193.08</v>
       </c>
-      <c r="G24" s="84">
+      <c r="G25" s="84">
         <v>157.88</v>
       </c>
-      <c r="H24" s="98">
-        <f>G24</f>
+      <c r="H25" s="98">
+        <f>G25</f>
         <v>157.88</v>
       </c>
-      <c r="I24" s="31">
-        <v>0</v>
-      </c>
-      <c r="J24" s="43">
+      <c r="I25" s="31">
+        <v>0</v>
+      </c>
+      <c r="J25" s="43">
         <v>503</v>
       </c>
-      <c r="K24" s="91">
+      <c r="K25" s="91">
         <v>0.91300000000000003</v>
       </c>
-      <c r="L24" s="92">
+      <c r="L25" s="92">
         <v>0.69099999999999995</v>
       </c>
-      <c r="M24" s="97">
-        <f t="shared" ref="M24" si="9">K24-L24</f>
+      <c r="M25" s="97">
+        <f t="shared" ref="M25" si="9">K25-L25</f>
         <v>0.22200000000000009</v>
       </c>
-      <c r="N24" s="92">
+      <c r="N25" s="92">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="O24" s="92">
+      <c r="O25" s="92">
         <v>4.2000000000000003E-2</v>
       </c>
-      <c r="P24" s="97">
-        <f t="shared" ref="P24" si="10">N24-O24</f>
+      <c r="P25" s="97">
+        <f t="shared" ref="P25" si="10">N25-O25</f>
         <v>-6.0000000000000053E-3</v>
       </c>
-      <c r="Q24" s="92">
+      <c r="Q25" s="92">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="R24" s="92">
+      <c r="R25" s="92">
         <v>0.26700000000000002</v>
       </c>
-      <c r="S24" s="97">
-        <f t="shared" ref="S24" si="11">Q24-R24</f>
+      <c r="S25" s="97">
+        <f t="shared" ref="S25" si="11">Q25-R25</f>
         <v>-0.21600000000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="E25" s="122"/>
-    </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A26" s="32" t="s">
-        <v>92</v>
+      <c r="A26" s="30" t="s">
+        <v>88</v>
       </c>
       <c r="C26" s="32" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E26" s="122"/>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A27" s="30"/>
-      <c r="B27" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="C27" s="37" t="s">
-        <v>86</v>
-      </c>
+      <c r="A27" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="E27" s="122"/>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
+      <c r="A28" s="30"/>
+      <c r="B28" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" s="37" t="s">
         <v>83</v>
-      </c>
-      <c r="B28" s="92">
-        <v>3.3696999999999999</v>
-      </c>
-      <c r="C28" s="118">
-        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="B29" s="108">
+        <v>80</v>
+      </c>
+      <c r="B29" s="92">
+        <v>3.3696999999999999</v>
+      </c>
+      <c r="C29" s="118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A30" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" s="108">
         <v>4.3080999999999996</v>
       </c>
-      <c r="C29" s="38">
+      <c r="C30" s="38">
         <v>9.7439999999999992E-3</v>
       </c>
     </row>
@@ -8540,12 +8555,12 @@
       <formula>0.45</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M20:M22">
+  <conditionalFormatting sqref="M20:M23">
     <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
       <formula>$M$19</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M24">
+  <conditionalFormatting sqref="M25">
     <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>

</xml_diff>

<commit_message>
Single-layer to 3-layer (1064nm)
Formatted to Opt. Commun.
</commit_message>
<xml_diff>
--- a/meetings/AsymReca_ThkCalc.xlsx
+++ b/meetings/AsymReca_ThkCalc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2024-ILLUSTRIOUS\My Drive (61050734@kmitl.ac.th)\AsymReca_SbSe\meetings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2930F64-1CFB-415C-91FC-D7054F5D9ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2FC23C-293D-4400-8BE6-65195114BC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="532" sheetId="8" r:id="rId1"/>
@@ -19,9 +19,10 @@
     <sheet name="800" sheetId="12" r:id="rId4"/>
     <sheet name="1064" sheetId="9" r:id="rId5"/>
     <sheet name="Amorphous phase" sheetId="7" state="hidden" r:id="rId6"/>
-    <sheet name="Crystalline" sheetId="4" r:id="rId7"/>
-    <sheet name="Sheet2" sheetId="5" state="hidden" r:id="rId8"/>
-    <sheet name="Sheet3" sheetId="6" state="hidden" r:id="rId9"/>
+    <sheet name="1064_back" sheetId="13" r:id="rId7"/>
+    <sheet name="Crystalline" sheetId="4" r:id="rId8"/>
+    <sheet name="Sheet2" sheetId="5" state="hidden" r:id="rId9"/>
+    <sheet name="Sheet3" sheetId="6" state="hidden" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="109">
   <si>
     <t>Wavelength (nm)</t>
   </si>
@@ -1903,6 +1904,39 @@
   </si>
   <si>
     <t>MaxT shifted to 1302</t>
+  </si>
+  <si>
+    <t>tH</t>
+  </si>
+  <si>
+    <t>TiO/SbSe/SiN</t>
+  </si>
+  <si>
+    <t>Broadband</t>
+  </si>
+  <si>
+    <t>SiN/SbSe/AlO</t>
+  </si>
+  <si>
+    <t>AlO/SbSe/MgF</t>
+  </si>
+  <si>
+    <t>SiO/SbSe/MgF</t>
+  </si>
+  <si>
+    <t>SbSe/Si/TiO</t>
+  </si>
+  <si>
+    <t>SbSe/TiO</t>
+  </si>
+  <si>
+    <t>non-QWOT</t>
+  </si>
+  <si>
+    <t>nS=SiO2</t>
+  </si>
+  <si>
+    <t>nS=nAir</t>
   </si>
 </sst>
 </file>
@@ -2263,7 +2297,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2632,17 +2666,50 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2650,34 +2717,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2686,15 +2729,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -2704,6 +2753,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -2713,11 +2768,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2731,41 +2804,14 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2773,7 +2819,17 @@
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="22">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2791,6 +2847,46 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3246,65 +3342,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="127" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="128" t="s">
+      <c r="C1" s="139" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="130" t="s">
+      <c r="E1" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="132" t="s">
+      <c r="F1" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="134" t="s">
+      <c r="G1" s="130" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="124" t="s">
+      <c r="H1" s="132" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="132" t="s">
+      <c r="I1" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="136" t="s">
+      <c r="J1" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="130" t="s">
+      <c r="K1" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="132"/>
+      <c r="L1" s="134"/>
       <c r="M1" s="138"/>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="132"/>
+      <c r="O1" s="134"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="130" t="s">
+      <c r="Q1" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="132"/>
+      <c r="R1" s="134"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="126" t="s">
+      <c r="T1" s="127" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="127"/>
+      <c r="A2" s="128"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="129"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="125"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="137"/>
+      <c r="C2" s="140"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="133"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="136"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -3332,11 +3428,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="127"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
+      <c r="T2" s="128"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -4604,6 +4700,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
@@ -4613,24 +4714,19 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:P1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="Q1:S1"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M18">
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="2" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M20:M21">
-    <cfRule type="cellIs" dxfId="15" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M40:M42">
-    <cfRule type="cellIs" dxfId="14" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="19" priority="4" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="5" operator="greaterThan">
@@ -4640,6 +4736,250 @@
   <hyperlinks>
     <hyperlink ref="A20" r:id="rId1" xr:uid="{0CA2BC15-2917-4413-A3B6-CA9BB1B2A39C}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37079731-60AB-4D94-B991-690660612702}">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="169" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="169" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="164" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="164" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="164" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="165" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="165"/>
+      <c r="H1" s="158" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="158"/>
+      <c r="J1" s="159" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="159"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="169"/>
+      <c r="B2" s="169"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="166" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="166">
+        <v>1320</v>
+      </c>
+      <c r="D3" s="166" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="3">
+        <v>100</v>
+      </c>
+      <c r="F3" s="10">
+        <v>0.23</v>
+      </c>
+      <c r="G3" s="10">
+        <v>0.05</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="167"/>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="167"/>
+      <c r="D4" s="168"/>
+      <c r="E4" s="1">
+        <v>100</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0.17</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="H4" s="8">
+        <v>0.15</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0.19</v>
+      </c>
+      <c r="J4" s="9">
+        <v>0.67</v>
+      </c>
+      <c r="K4" s="9">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="167"/>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="167"/>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="2">
+        <f>3.5*2</f>
+        <v>7</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.41</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0.08</v>
+      </c>
+      <c r="H5" s="5">
+        <v>0.59</v>
+      </c>
+      <c r="I5" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="167"/>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="167"/>
+      <c r="D6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="2">
+        <f>13.9*2</f>
+        <v>27.8</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="H6" s="5">
+        <v>0.83</v>
+      </c>
+      <c r="I6" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="168"/>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="168"/>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2">
+        <f>8.5*2</f>
+        <v>17</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.38</v>
+      </c>
+      <c r="G7" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0.62</v>
+      </c>
+      <c r="I7" s="5">
+        <v>0.39</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0.54</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4672,65 +5012,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="127" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="140" t="s">
+      <c r="C1" s="143" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="130" t="s">
+      <c r="E1" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="132" t="s">
+      <c r="F1" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="134" t="s">
+      <c r="G1" s="130" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="139" t="s">
+      <c r="H1" s="142" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="132" t="s">
+      <c r="I1" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="136" t="s">
+      <c r="J1" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="130" t="s">
+      <c r="K1" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="132"/>
+      <c r="L1" s="134"/>
       <c r="M1" s="138"/>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="132"/>
+      <c r="O1" s="134"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="130" t="s">
+      <c r="Q1" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="132"/>
+      <c r="R1" s="134"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="126" t="s">
+      <c r="T1" s="127" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="127"/>
+      <c r="A2" s="128"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="141"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="137"/>
+      <c r="C2" s="144"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="128"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="136"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -4758,11 +5098,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="127"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
+      <c r="T2" s="128"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -5685,6 +6025,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -5693,21 +6039,15 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M4:M17">
-    <cfRule type="cellIs" dxfId="13" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="12" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -5746,65 +6086,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="127" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="140" t="s">
+      <c r="C1" s="143" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="130" t="s">
+      <c r="E1" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="132" t="s">
+      <c r="F1" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="134" t="s">
+      <c r="G1" s="130" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="139" t="s">
+      <c r="H1" s="142" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="132" t="s">
+      <c r="I1" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="136" t="s">
+      <c r="J1" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="130" t="s">
+      <c r="K1" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="132"/>
+      <c r="L1" s="134"/>
       <c r="M1" s="138"/>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="132"/>
+      <c r="O1" s="134"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="130" t="s">
+      <c r="Q1" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="132"/>
+      <c r="R1" s="134"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="126" t="s">
+      <c r="T1" s="127" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="127"/>
+      <c r="A2" s="128"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="141"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="137"/>
+      <c r="C2" s="144"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="128"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="136"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -5832,11 +6172,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="127"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
+      <c r="T2" s="128"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -6500,6 +6840,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -6508,20 +6854,14 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M12">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -6560,65 +6900,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="127" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="140" t="s">
+      <c r="C1" s="143" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="130" t="s">
+      <c r="E1" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="132" t="s">
+      <c r="F1" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="134" t="s">
+      <c r="G1" s="130" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="139" t="s">
+      <c r="H1" s="142" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="132" t="s">
+      <c r="I1" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="136" t="s">
+      <c r="J1" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="130" t="s">
+      <c r="K1" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="132"/>
+      <c r="L1" s="134"/>
       <c r="M1" s="138"/>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="132"/>
+      <c r="O1" s="134"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="130" t="s">
+      <c r="Q1" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="132"/>
+      <c r="R1" s="134"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="126" t="s">
+      <c r="T1" s="127" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="127"/>
+      <c r="A2" s="128"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="141"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="137"/>
+      <c r="C2" s="144"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="128"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="136"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -6646,11 +6986,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="127"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
+      <c r="T2" s="128"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -7193,12 +7533,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -7207,14 +7541,20 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M7 M10:M11">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -7253,65 +7593,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="127" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="128" t="s">
+      <c r="C1" s="139" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="130" t="s">
+      <c r="E1" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="132" t="s">
+      <c r="F1" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="134" t="s">
+      <c r="G1" s="130" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="124" t="s">
+      <c r="H1" s="132" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="132" t="s">
+      <c r="I1" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="136" t="s">
+      <c r="J1" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="130" t="s">
+      <c r="K1" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="132"/>
+      <c r="L1" s="134"/>
       <c r="M1" s="138"/>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="132"/>
+      <c r="O1" s="134"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="130" t="s">
+      <c r="Q1" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="132"/>
+      <c r="R1" s="134"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="166" t="s">
+      <c r="T1" s="145" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="127"/>
+      <c r="A2" s="128"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="129"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="125"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="137"/>
+      <c r="C2" s="140"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="133"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="136"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -7339,11 +7679,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="167"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
+      <c r="T2" s="146"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -7395,7 +7735,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
       <c r="P3" s="90">
-        <f t="shared" ref="P3:P6" si="1">N3-O3</f>
+        <f>N3-O3</f>
         <v>-1.2999999999999666E-2</v>
       </c>
       <c r="Q3" s="96">
@@ -7405,7 +7745,7 @@
         <v>0.7</v>
       </c>
       <c r="S3" s="90">
-        <f t="shared" ref="S3:S6" si="2">Q3-R3</f>
+        <f t="shared" ref="S3:S6" si="1">Q3-R3</f>
         <v>-0.7</v>
       </c>
       <c r="T3" s="35" t="s">
@@ -7458,7 +7798,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="P4" s="97">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="P3:P6" si="2">N4-O4</f>
         <v>-1.5000000000000444E-2</v>
       </c>
       <c r="Q4" s="92">
@@ -7468,8 +7808,11 @@
         <v>0.44</v>
       </c>
       <c r="S4" s="97">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-0.44</v>
+      </c>
+      <c r="T4" s="35" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
@@ -7518,7 +7861,7 @@
         <v>1.2E-2</v>
       </c>
       <c r="P5" s="97">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1.199999999999889E-2</v>
       </c>
       <c r="Q5" s="92">
@@ -7528,7 +7871,7 @@
         <v>0.72199999999999998</v>
       </c>
       <c r="S5" s="97">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-0.72199999999999998</v>
       </c>
       <c r="T5" s="71"/>
@@ -7579,7 +7922,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="P6" s="97">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-8.0000000000000002E-3</v>
       </c>
       <c r="Q6" s="92">
@@ -7589,7 +7932,7 @@
         <v>0.89600000000000002</v>
       </c>
       <c r="S6" s="97">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-0.89600000000000002</v>
       </c>
       <c r="T6" s="71"/>
@@ -7928,7 +8271,7 @@
         <v>49.7</v>
       </c>
       <c r="H14" s="98">
-        <f t="shared" ref="H14:H18" si="8">G14</f>
+        <f t="shared" ref="H14:H17" si="8">G14</f>
         <v>49.7</v>
       </c>
       <c r="I14" s="84">
@@ -8212,8 +8555,8 @@
         <f>R19-Q19</f>
         <v>-0.48499999999999999</v>
       </c>
-      <c r="T19" s="168">
-        <v>597</v>
+      <c r="T19" s="126" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
@@ -8403,7 +8746,7 @@
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="C23" s="165"/>
+      <c r="C23" s="125"/>
       <c r="M23" s="97"/>
       <c r="P23" s="97"/>
       <c r="S23" s="97"/>
@@ -8415,8 +8758,61 @@
       <c r="B24" s="32">
         <v>0</v>
       </c>
+      <c r="C24" s="32" t="s">
+        <v>74</v>
+      </c>
       <c r="D24" s="38">
         <v>0</v>
+      </c>
+      <c r="E24" s="44">
+        <v>0</v>
+      </c>
+      <c r="F24" s="34">
+        <v>0</v>
+      </c>
+      <c r="G24" s="84">
+        <v>157.88</v>
+      </c>
+      <c r="H24" s="98">
+        <f>G24</f>
+        <v>157.88</v>
+      </c>
+      <c r="I24" s="31">
+        <v>0</v>
+      </c>
+      <c r="J24" s="43">
+        <f>G24</f>
+        <v>157.88</v>
+      </c>
+      <c r="K24" s="91">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="L24" s="92">
+        <v>0.38</v>
+      </c>
+      <c r="M24" s="97">
+        <f t="shared" ref="M24" si="9">K24-L24</f>
+        <v>0.58399999999999996</v>
+      </c>
+      <c r="N24" s="92">
+        <v>0</v>
+      </c>
+      <c r="O24" s="92">
+        <v>1.2E-2</v>
+      </c>
+      <c r="P24" s="97">
+        <f t="shared" ref="P24" si="10">N24-O24</f>
+        <v>-1.2E-2</v>
+      </c>
+      <c r="Q24" s="92">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="R24" s="92">
+        <v>0.60799999999999998</v>
+      </c>
+      <c r="S24" s="97">
+        <f t="shared" ref="S24" si="11">Q24-R24</f>
+        <v>-0.57199999999999995</v>
       </c>
     </row>
     <row r="25" spans="1:20" ht="22.5" x14ac:dyDescent="0.25">
@@ -8452,7 +8848,7 @@
         <v>0.69099999999999995</v>
       </c>
       <c r="M25" s="97">
-        <f t="shared" ref="M25" si="9">K25-L25</f>
+        <f t="shared" ref="M25" si="12">K25-L25</f>
         <v>0.22200000000000009</v>
       </c>
       <c r="N25" s="92">
@@ -8462,7 +8858,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
       <c r="P25" s="97">
-        <f t="shared" ref="P25" si="10">N25-O25</f>
+        <f t="shared" ref="P25" si="13">N25-O25</f>
         <v>-6.0000000000000053E-3</v>
       </c>
       <c r="Q25" s="92">
@@ -8472,7 +8868,7 @@
         <v>0.26700000000000002</v>
       </c>
       <c r="S25" s="97">
-        <f t="shared" ref="S25" si="11">Q25-R25</f>
+        <f t="shared" ref="S25" si="14">Q25-R25</f>
         <v>-0.21600000000000003</v>
       </c>
     </row>
@@ -8527,6 +8923,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="I1:I2"/>
@@ -8535,33 +8937,32 @@
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M17 M19">
-    <cfRule type="cellIs" dxfId="7" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="5" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M16:M18">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="6" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" priority="7" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M20:M23">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
       <formula>$M$19</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M25">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="greaterThan">
+      <formula>$M$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M24">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8597,66 +8998,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="126" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="147" t="s">
+      <c r="B1" s="127" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="152" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="128" t="s">
+      <c r="D1" s="139" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="130" t="s">
+      <c r="E1" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="132" t="s">
+      <c r="F1" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="139" t="s">
+      <c r="G1" s="142" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="139" t="s">
+      <c r="H1" s="142" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="132" t="s">
+      <c r="I1" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="136" t="s">
+      <c r="J1" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="130" t="s">
+      <c r="K1" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="132"/>
+      <c r="L1" s="134"/>
       <c r="M1" s="138"/>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="132"/>
+      <c r="O1" s="134"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="130" t="s">
+      <c r="Q1" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="132"/>
+      <c r="R1" s="134"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="146" t="s">
+      <c r="T1" s="151" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="133"/>
-      <c r="B2" s="127"/>
-      <c r="C2" s="141"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="137"/>
+      <c r="A2" s="129"/>
+      <c r="B2" s="128"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="128"/>
+      <c r="H2" s="128"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="136"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -8684,11 +9085,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="133"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
+      <c r="T2" s="129"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="46">
@@ -8758,16 +9159,16 @@
       <c r="D4" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="143">
+      <c r="E4" s="147">
         <v>32.700000000000003</v>
       </c>
-      <c r="F4" s="144">
+      <c r="F4" s="148">
         <v>90.1</v>
       </c>
-      <c r="G4" s="145">
+      <c r="G4" s="150">
         <v>38.5</v>
       </c>
-      <c r="H4" s="145"/>
+      <c r="H4" s="150"/>
       <c r="I4" s="66">
         <v>18.3</v>
       </c>
@@ -8810,12 +9211,12 @@
       <c r="D5" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="143"/>
-      <c r="F5" s="144"/>
-      <c r="G5" s="142">
+      <c r="E5" s="147"/>
+      <c r="F5" s="148"/>
+      <c r="G5" s="149">
         <v>41.2</v>
       </c>
-      <c r="H5" s="142"/>
+      <c r="H5" s="149"/>
       <c r="I5" s="58">
         <v>15.1</v>
       </c>
@@ -8860,12 +9261,12 @@
       <c r="D6" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="143"/>
-      <c r="F6" s="144"/>
-      <c r="G6" s="142">
+      <c r="E6" s="147"/>
+      <c r="F6" s="148"/>
+      <c r="G6" s="149">
         <v>24.3</v>
       </c>
-      <c r="H6" s="142"/>
+      <c r="H6" s="149"/>
       <c r="I6" s="58">
         <v>30.6</v>
       </c>
@@ -8907,12 +9308,12 @@
       <c r="D7" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="143"/>
-      <c r="F7" s="144"/>
-      <c r="G7" s="142">
+      <c r="E7" s="147"/>
+      <c r="F7" s="148"/>
+      <c r="G7" s="149">
         <v>42.6</v>
       </c>
-      <c r="H7" s="142"/>
+      <c r="H7" s="149"/>
       <c r="I7" s="58">
         <v>13.3</v>
       </c>
@@ -8956,12 +9357,12 @@
       <c r="D8" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="143"/>
-      <c r="F8" s="144"/>
-      <c r="G8" s="142">
+      <c r="E8" s="147"/>
+      <c r="F8" s="148"/>
+      <c r="G8" s="149">
         <v>31.9</v>
       </c>
-      <c r="H8" s="142"/>
+      <c r="H8" s="149"/>
       <c r="I8" s="58">
         <v>23.7</v>
       </c>
@@ -9003,8 +9404,8 @@
       <c r="D9" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="143"/>
-      <c r="F9" s="144"/>
+      <c r="E9" s="147"/>
+      <c r="F9" s="148"/>
       <c r="G9" s="66">
         <v>2.7</v>
       </c>
@@ -9053,8 +9454,8 @@
       <c r="D10" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="143"/>
-      <c r="F10" s="144"/>
+      <c r="E10" s="147"/>
+      <c r="F10" s="148"/>
       <c r="G10" s="58">
         <v>4.2</v>
       </c>
@@ -9103,8 +9504,8 @@
       <c r="D11" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="143"/>
-      <c r="F11" s="144"/>
+      <c r="E11" s="147"/>
+      <c r="F11" s="148"/>
       <c r="G11" s="58">
         <v>1.3</v>
       </c>
@@ -9222,16 +9623,16 @@
       <c r="D14" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="143">
+      <c r="E14" s="147">
         <v>66.599999999999994</v>
       </c>
-      <c r="F14" s="144">
+      <c r="F14" s="148">
         <v>181.3</v>
       </c>
-      <c r="G14" s="142">
+      <c r="G14" s="149">
         <v>107.3</v>
       </c>
-      <c r="H14" s="142"/>
+      <c r="H14" s="149"/>
       <c r="I14" s="58">
         <v>0</v>
       </c>
@@ -9273,12 +9674,12 @@
       <c r="D15" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="143"/>
-      <c r="F15" s="144"/>
-      <c r="G15" s="145">
+      <c r="E15" s="147"/>
+      <c r="F15" s="148"/>
+      <c r="G15" s="150">
         <v>68.7</v>
       </c>
-      <c r="H15" s="145"/>
+      <c r="H15" s="150"/>
       <c r="I15" s="66">
         <v>51.9</v>
       </c>
@@ -9321,12 +9722,12 @@
       <c r="D16" s="81" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="143"/>
-      <c r="F16" s="144"/>
-      <c r="G16" s="145">
+      <c r="E16" s="147"/>
+      <c r="F16" s="148"/>
+      <c r="G16" s="150">
         <v>105</v>
       </c>
-      <c r="H16" s="145"/>
+      <c r="H16" s="150"/>
       <c r="I16" s="66">
         <v>0</v>
       </c>
@@ -9369,12 +9770,12 @@
       <c r="D17" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="143"/>
-      <c r="F17" s="144"/>
-      <c r="G17" s="142">
+      <c r="E17" s="147"/>
+      <c r="F17" s="148"/>
+      <c r="G17" s="149">
         <v>65.599999999999994</v>
       </c>
-      <c r="H17" s="142"/>
+      <c r="H17" s="149"/>
       <c r="I17" s="58">
         <v>53.5</v>
       </c>
@@ -9417,8 +9818,8 @@
       <c r="D18" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="143"/>
-      <c r="F18" s="144"/>
+      <c r="E18" s="147"/>
+      <c r="F18" s="148"/>
       <c r="G18" s="58">
         <v>42.6</v>
       </c>
@@ -9467,8 +9868,8 @@
       <c r="D19" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="143"/>
-      <c r="F19" s="144"/>
+      <c r="E19" s="147"/>
+      <c r="F19" s="148"/>
       <c r="G19" s="58">
         <v>47.7</v>
       </c>
@@ -9517,8 +9918,8 @@
       <c r="D20" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="143"/>
-      <c r="F20" s="144"/>
+      <c r="E20" s="147"/>
+      <c r="F20" s="148"/>
       <c r="G20" s="58">
         <v>48.7</v>
       </c>
@@ -9674,12 +10075,18 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="E14:E20"/>
-    <mergeCell ref="F14:F20"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="E4:E11"/>
+    <mergeCell ref="F4:F11"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="N1:P1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
@@ -9691,26 +10098,20 @@
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="E4:E11"/>
-    <mergeCell ref="F4:F11"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E14:E20"/>
+    <mergeCell ref="F14:F20"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G14:H14"/>
   </mergeCells>
   <conditionalFormatting sqref="M14:M20">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>$M$13</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M29:M33">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -9722,6 +10123,660 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6C66A9-86C5-4B44-B720-CA86E494EFA2}">
+  <dimension ref="A1:W28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" style="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="35" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" style="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" style="38" customWidth="1"/>
+    <col min="5" max="5" width="7.7109375" style="108" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" style="44" customWidth="1"/>
+    <col min="7" max="7" width="7.7109375" style="34" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" style="84" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" style="43" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" style="91" customWidth="1"/>
+    <col min="11" max="11" width="7.28515625" style="92" customWidth="1"/>
+    <col min="12" max="12" width="7.28515625" style="41" customWidth="1"/>
+    <col min="13" max="14" width="7.28515625" style="92" customWidth="1"/>
+    <col min="15" max="15" width="7.28515625" style="41" customWidth="1"/>
+    <col min="16" max="17" width="7.28515625" style="92" customWidth="1"/>
+    <col min="18" max="18" width="7.28515625" style="41" customWidth="1"/>
+    <col min="19" max="23" width="7.28515625" style="32" customWidth="1"/>
+    <col min="24" max="16384" width="9.140625" style="32"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="127" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="145" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="139" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="170" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="137" t="s">
+        <v>98</v>
+      </c>
+      <c r="G1" s="134" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" s="137" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="134"/>
+      <c r="L1" s="138"/>
+      <c r="M1" s="137" t="s">
+        <v>4</v>
+      </c>
+      <c r="N1" s="134"/>
+      <c r="O1" s="138"/>
+      <c r="P1" s="137" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q1" s="134"/>
+      <c r="R1" s="138"/>
+    </row>
+    <row r="2" spans="1:23" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="128"/>
+      <c r="B2" s="146"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="124"/>
+      <c r="F2" s="141"/>
+      <c r="G2" s="129"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="136"/>
+      <c r="J2" s="111" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="O2" s="52" t="s">
+        <v>50</v>
+      </c>
+      <c r="P2" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" s="52" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" s="129"/>
+      <c r="U2" s="129"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+    </row>
+    <row r="3" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="30">
+        <v>1064</v>
+      </c>
+      <c r="B3" s="35"/>
+      <c r="C3" s="45" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="37"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="84">
+        <v>157.86000000000001</v>
+      </c>
+      <c r="I3" s="83">
+        <f>H3</f>
+        <v>157.86000000000001</v>
+      </c>
+      <c r="J3" s="95">
+        <v>0.93100000000000005</v>
+      </c>
+      <c r="K3" s="96">
+        <v>0.374</v>
+      </c>
+      <c r="L3" s="90">
+        <f t="shared" ref="L3:L9" si="0">J3-K3</f>
+        <v>0.55700000000000005</v>
+      </c>
+      <c r="M3" s="96">
+        <v>0</v>
+      </c>
+      <c r="N3" s="96">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="O3" s="90">
+        <f t="shared" ref="O3:O9" si="1">M3-N3</f>
+        <v>-1.2999999999999999E-2</v>
+      </c>
+      <c r="P3" s="96">
+        <v>6.9000000000000006E-2</v>
+      </c>
+      <c r="Q3" s="96">
+        <v>0.61299999999999999</v>
+      </c>
+      <c r="R3" s="90">
+        <f t="shared" ref="R3:R7" si="2">P3-Q3</f>
+        <v>-0.54400000000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C4" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="F4" s="44">
+        <v>115.17</v>
+      </c>
+      <c r="H4" s="84">
+        <v>78.930000000000007</v>
+      </c>
+      <c r="I4" s="43">
+        <f>F4+H4</f>
+        <v>194.10000000000002</v>
+      </c>
+      <c r="J4" s="91">
+        <v>0.93300000000000005</v>
+      </c>
+      <c r="K4" s="92">
+        <v>0.77100000000000002</v>
+      </c>
+      <c r="L4" s="90">
+        <f t="shared" si="0"/>
+        <v>0.16200000000000003</v>
+      </c>
+      <c r="M4" s="92">
+        <v>0</v>
+      </c>
+      <c r="N4" s="92">
+        <v>0.01</v>
+      </c>
+      <c r="O4" s="90">
+        <f t="shared" si="1"/>
+        <v>-0.01</v>
+      </c>
+      <c r="P4" s="92">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="Q4" s="92">
+        <v>0.219</v>
+      </c>
+      <c r="R4" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B5" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="44">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="H5" s="84">
+        <v>162</v>
+      </c>
+      <c r="I5" s="43">
+        <f>F5+H5</f>
+        <v>194.8</v>
+      </c>
+      <c r="J5" s="91">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="K5" s="92">
+        <v>0.83</v>
+      </c>
+      <c r="L5" s="90">
+        <f t="shared" si="0"/>
+        <v>0.13400000000000001</v>
+      </c>
+      <c r="M5" s="92">
+        <v>0</v>
+      </c>
+      <c r="N5" s="92">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="O5" s="90">
+        <f t="shared" si="1"/>
+        <v>-8.0000000000000002E-3</v>
+      </c>
+      <c r="P5" s="92">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="Q5" s="92">
+        <v>0.16200000000000001</v>
+      </c>
+      <c r="R5" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B6" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="F6" s="172">
+        <v>68.25</v>
+      </c>
+      <c r="H6" s="84">
+        <v>125</v>
+      </c>
+      <c r="I6" s="43">
+        <f>F6+H6</f>
+        <v>193.25</v>
+      </c>
+      <c r="J6" s="91">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="K6" s="92">
+        <v>0.70099999999999996</v>
+      </c>
+      <c r="L6" s="90">
+        <f t="shared" si="0"/>
+        <v>0.26300000000000001</v>
+      </c>
+      <c r="M6" s="92">
+        <v>0</v>
+      </c>
+      <c r="N6" s="92">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="O6" s="90">
+        <f t="shared" si="1"/>
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="P6" s="92">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="Q6" s="92">
+        <v>0.28100000000000003</v>
+      </c>
+      <c r="R6" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.24500000000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="C7" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="44">
+        <v>136.35</v>
+      </c>
+      <c r="G7" s="34">
+        <v>115.17</v>
+      </c>
+      <c r="H7" s="84">
+        <v>78.930000000000007</v>
+      </c>
+      <c r="I7" s="43">
+        <f>SUM(F7:H7)</f>
+        <v>330.45</v>
+      </c>
+      <c r="J7" s="91">
+        <v>0.93300000000000005</v>
+      </c>
+      <c r="K7" s="92">
+        <v>0.77100000000000002</v>
+      </c>
+      <c r="L7" s="90">
+        <f t="shared" si="0"/>
+        <v>0.16200000000000003</v>
+      </c>
+      <c r="M7" s="92">
+        <v>0</v>
+      </c>
+      <c r="N7" s="92">
+        <v>0.01</v>
+      </c>
+      <c r="O7" s="90">
+        <f t="shared" si="1"/>
+        <v>-0.01</v>
+      </c>
+      <c r="P7" s="92">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="Q7" s="92">
+        <v>0.218</v>
+      </c>
+      <c r="R7" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="30"/>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="30"/>
+      <c r="D10" s="37"/>
+      <c r="L10" s="97"/>
+      <c r="O10" s="97"/>
+      <c r="R10" s="97"/>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B11" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="F11" s="44">
+        <v>181.31</v>
+      </c>
+      <c r="G11" s="34">
+        <v>193.08</v>
+      </c>
+      <c r="H11" s="84">
+        <v>157.86000000000001</v>
+      </c>
+      <c r="I11" s="43">
+        <f>SUM(F11:H11)</f>
+        <v>532.25</v>
+      </c>
+      <c r="J11" s="91">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="K11" s="92">
+        <v>0.56100000000000005</v>
+      </c>
+      <c r="L11" s="90">
+        <f>J11-K11</f>
+        <v>0.3879999999999999</v>
+      </c>
+      <c r="M11" s="92">
+        <v>0</v>
+      </c>
+      <c r="N11" s="92">
+        <v>1.9E-2</v>
+      </c>
+      <c r="O11" s="90">
+        <f>M11-N11</f>
+        <v>-1.9E-2</v>
+      </c>
+      <c r="P11" s="92">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="Q11" s="92">
+        <v>0.42</v>
+      </c>
+      <c r="R11" s="90">
+        <f>P11-Q11</f>
+        <v>-0.36899999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B12" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" s="44">
+        <v>164.55</v>
+      </c>
+      <c r="G12" s="34">
+        <v>193.08</v>
+      </c>
+      <c r="H12" s="84">
+        <v>157.86000000000001</v>
+      </c>
+      <c r="I12" s="43">
+        <f>SUM(F12:H12)</f>
+        <v>515.49</v>
+      </c>
+      <c r="J12" s="91">
+        <v>0.96299999999999997</v>
+      </c>
+      <c r="K12" s="92">
+        <v>0.623</v>
+      </c>
+      <c r="L12" s="90">
+        <f>J12-K12</f>
+        <v>0.33999999999999997</v>
+      </c>
+      <c r="M12" s="92">
+        <v>0</v>
+      </c>
+      <c r="N12" s="92">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="O12" s="90">
+        <f>M12-N12</f>
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="P12" s="92">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="Q12" s="92">
+        <v>0.35899999999999999</v>
+      </c>
+      <c r="R12" s="90">
+        <f>P12-Q12</f>
+        <v>-0.32200000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B13" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="37"/>
+      <c r="F13" s="44">
+        <v>133.22999999999999</v>
+      </c>
+      <c r="G13" s="34">
+        <v>164.55</v>
+      </c>
+      <c r="H13" s="84">
+        <v>157.86000000000001</v>
+      </c>
+      <c r="I13" s="43">
+        <f>SUM(F13:H13)</f>
+        <v>455.64</v>
+      </c>
+      <c r="J13" s="91">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="K13" s="92">
+        <v>0.82899999999999996</v>
+      </c>
+      <c r="L13" s="90">
+        <f>J13-K13</f>
+        <v>0.13500000000000001</v>
+      </c>
+      <c r="M13" s="92">
+        <v>0</v>
+      </c>
+      <c r="N13" s="92">
+        <v>1.9E-2</v>
+      </c>
+      <c r="O13" s="90">
+        <f>M13-N13</f>
+        <v>-1.9E-2</v>
+      </c>
+      <c r="P13" s="92">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="Q13" s="92">
+        <v>0.152</v>
+      </c>
+      <c r="R13" s="90">
+        <f>P13-Q13</f>
+        <v>-0.11599999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B14" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="F14" s="44">
+        <v>115.17</v>
+      </c>
+      <c r="G14" s="34">
+        <v>133.22999999999999</v>
+      </c>
+      <c r="H14" s="84">
+        <v>157.86000000000001</v>
+      </c>
+      <c r="I14" s="43">
+        <f>SUM(F14:H14)</f>
+        <v>406.26</v>
+      </c>
+      <c r="J14" s="91">
+        <v>0.96199999999999997</v>
+      </c>
+      <c r="K14" s="92">
+        <v>0.93799999999999994</v>
+      </c>
+      <c r="L14" s="90">
+        <f>J14-K14</f>
+        <v>2.4000000000000021E-2</v>
+      </c>
+      <c r="M14" s="92">
+        <v>0</v>
+      </c>
+      <c r="N14" s="92">
+        <v>1.9E-2</v>
+      </c>
+      <c r="O14" s="90">
+        <f>M14-N14</f>
+        <v>-1.9E-2</v>
+      </c>
+      <c r="P14" s="92">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="Q14" s="92">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="R14" s="90">
+        <f>P14-Q14</f>
+        <v>-4.9999999999999975E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B18" s="71"/>
+      <c r="L18" s="97"/>
+      <c r="O18" s="97"/>
+      <c r="R18" s="97"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B19" s="71"/>
+      <c r="L19" s="97"/>
+      <c r="O19" s="97"/>
+      <c r="R19" s="97"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L20" s="97"/>
+      <c r="O20" s="97"/>
+      <c r="R20" s="97"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L21" s="97"/>
+      <c r="O21" s="97"/>
+      <c r="R21" s="97"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="C23" s="37"/>
+      <c r="F23" s="122"/>
+      <c r="L23" s="97"/>
+      <c r="O23" s="97"/>
+      <c r="R23" s="97"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" s="30"/>
+      <c r="F24" s="122"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="F25" s="122"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A26" s="30"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" s="30"/>
+      <c r="C27" s="118"/>
+      <c r="D27" s="171"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="B1:B2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="L10:L17">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+      <formula>$L$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L16:L17">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
+      <formula>0.45</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="greaterThan">
+      <formula>0.45</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L18:L21">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L23">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+      <formula>$L$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03EBE129-7102-4E9D-8A3D-9B26EFEE1948}">
   <dimension ref="A1:Y21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9749,66 +10804,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="126" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="147" t="s">
+      <c r="B1" s="127" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="152" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="128" t="s">
+      <c r="D1" s="139" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="130" t="s">
+      <c r="E1" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="132" t="s">
+      <c r="F1" s="134" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="139" t="s">
+      <c r="G1" s="142" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="139" t="s">
+      <c r="H1" s="142" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="132" t="s">
+      <c r="I1" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="136" t="s">
+      <c r="J1" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="130" t="s">
+      <c r="K1" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="132"/>
+      <c r="L1" s="134"/>
       <c r="M1" s="138"/>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="132"/>
+      <c r="O1" s="134"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="130" t="s">
+      <c r="Q1" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="132"/>
+      <c r="R1" s="134"/>
       <c r="S1" s="138"/>
-      <c r="T1" s="151" t="s">
+      <c r="T1" s="153" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="133"/>
-      <c r="B2" s="127"/>
-      <c r="C2" s="141"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="137"/>
+      <c r="A2" s="129"/>
+      <c r="B2" s="128"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="128"/>
+      <c r="H2" s="128"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="136"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -9836,11 +10891,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="152"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
+      <c r="T2" s="154"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="30">
@@ -9852,10 +10907,10 @@
       <c r="D3" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="148">
-        <v>0</v>
-      </c>
-      <c r="F3" s="150">
+      <c r="E3" s="155">
+        <v>0</v>
+      </c>
+      <c r="F3" s="157">
         <v>0</v>
       </c>
       <c r="G3" s="58">
@@ -9907,8 +10962,8 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E4" s="149"/>
-      <c r="F4" s="142"/>
+      <c r="E4" s="156"/>
+      <c r="F4" s="149"/>
       <c r="G4" s="58">
         <v>35.6</v>
       </c>
@@ -9961,10 +11016,10 @@
       <c r="D5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="143">
+      <c r="E5" s="147">
         <v>32.700000000000003</v>
       </c>
-      <c r="F5" s="144">
+      <c r="F5" s="148">
         <v>90.1</v>
       </c>
       <c r="G5" s="58">
@@ -10017,8 +11072,8 @@
       <c r="D6" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="143"/>
-      <c r="F6" s="144"/>
+      <c r="E6" s="147"/>
+      <c r="F6" s="148"/>
       <c r="G6" s="58">
         <v>35.6</v>
       </c>
@@ -10141,10 +11196,10 @@
       <c r="D9" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="143">
+      <c r="E9" s="147">
         <v>66.599999999999994</v>
       </c>
-      <c r="F9" s="144">
+      <c r="F9" s="148">
         <v>181.3</v>
       </c>
       <c r="G9" s="58">
@@ -10196,8 +11251,8 @@
       <c r="D10" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="143"/>
-      <c r="F10" s="144"/>
+      <c r="E10" s="147"/>
+      <c r="F10" s="148"/>
       <c r="G10" s="58">
         <v>75.8</v>
       </c>
@@ -10247,8 +11302,8 @@
       <c r="D11" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="143"/>
-      <c r="F11" s="144"/>
+      <c r="E11" s="147"/>
+      <c r="F11" s="148"/>
       <c r="G11" s="58">
         <v>89.5</v>
       </c>
@@ -10296,8 +11351,8 @@
       <c r="D12" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="143"/>
-      <c r="F12" s="144"/>
+      <c r="E12" s="147"/>
+      <c r="F12" s="148"/>
       <c r="G12" s="58">
         <v>46.1</v>
       </c>
@@ -10347,8 +11402,8 @@
       <c r="D13" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="143"/>
-      <c r="F13" s="144"/>
+      <c r="E13" s="147"/>
+      <c r="F13" s="148"/>
       <c r="G13" s="58">
         <v>73.400000000000006</v>
       </c>
@@ -10397,8 +11452,8 @@
       <c r="D14" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="143"/>
-      <c r="F14" s="144"/>
+      <c r="E14" s="147"/>
+      <c r="F14" s="148"/>
       <c r="G14" s="58">
         <v>88.4</v>
       </c>
@@ -10447,8 +11502,8 @@
       <c r="D15" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="143"/>
-      <c r="F15" s="144"/>
+      <c r="E15" s="147"/>
+      <c r="F15" s="148"/>
       <c r="G15" s="58">
         <v>27.5</v>
       </c>
@@ -10497,8 +11552,8 @@
       <c r="D16" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="143"/>
-      <c r="F16" s="144"/>
+      <c r="E16" s="147"/>
+      <c r="F16" s="148"/>
       <c r="G16" s="58">
         <v>94.8</v>
       </c>
@@ -10547,8 +11602,8 @@
       <c r="D17" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="143"/>
-      <c r="F17" s="144"/>
+      <c r="E17" s="147"/>
+      <c r="F17" s="148"/>
       <c r="G17" s="58">
         <v>861.6</v>
       </c>
@@ -10600,8 +11655,8 @@
       <c r="D18" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="143"/>
-      <c r="F18" s="144"/>
+      <c r="E18" s="147"/>
+      <c r="F18" s="148"/>
       <c r="G18" s="58">
         <v>48.1</v>
       </c>
@@ -10650,8 +11705,8 @@
       <c r="D19" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="143"/>
-      <c r="F19" s="144"/>
+      <c r="E19" s="147"/>
+      <c r="F19" s="148"/>
       <c r="G19" s="58">
         <v>41.8</v>
       </c>
@@ -10706,14 +11761,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:P1"/>
     <mergeCell ref="E9:E19"/>
     <mergeCell ref="F9:F19"/>
     <mergeCell ref="B1:B2"/>
@@ -10728,10 +11775,18 @@
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M9:M19">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -10739,7 +11794,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M9:M20">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>$M$8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10747,7 +11802,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BF2213B-BB65-498C-AA64-42693820505C}">
   <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -10761,25 +11816,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="156" t="s">
+      <c r="A1" s="169" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="156" t="s">
+      <c r="B1" s="169" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="157" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="157" t="s">
+      <c r="C1" s="164" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="164" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="157" t="s">
+      <c r="E1" s="164" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="164" t="s">
+      <c r="F1" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="164"/>
+      <c r="G1" s="165"/>
       <c r="H1" s="158" t="s">
         <v>4</v>
       </c>
@@ -10790,11 +11845,11 @@
       <c r="K1" s="159"/>
     </row>
     <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="156"/>
-      <c r="B2" s="156"/>
-      <c r="C2" s="157"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="157"/>
+      <c r="A2" s="169"/>
+      <c r="B2" s="169"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
       <c r="F2" s="14" t="s">
         <v>7</v>
       </c>
@@ -10943,16 +11998,16 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="153" t="s">
+      <c r="A7" s="166" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="153">
+      <c r="C7" s="166">
         <v>1320</v>
       </c>
-      <c r="D7" s="153" t="s">
+      <c r="D7" s="166" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="3">
@@ -10978,12 +12033,12 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="154"/>
+      <c r="A8" s="167"/>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="154"/>
-      <c r="D8" s="155"/>
+      <c r="C8" s="167"/>
+      <c r="D8" s="168"/>
       <c r="E8" s="1">
         <v>100</v>
       </c>
@@ -11007,11 +12062,11 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="154"/>
+      <c r="A9" s="167"/>
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="154"/>
+      <c r="C9" s="167"/>
       <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
@@ -11039,11 +12094,11 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="154"/>
+      <c r="A10" s="167"/>
       <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="154"/>
+      <c r="C10" s="167"/>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
@@ -11071,11 +12126,11 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="155"/>
+      <c r="A11" s="168"/>
       <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="155"/>
+      <c r="C11" s="168"/>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
@@ -11104,6 +12159,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="C3:C6"/>
@@ -11111,257 +12173,6 @@
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37079731-60AB-4D94-B991-690660612702}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="156" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="156" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="157" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="157" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="157" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="164" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="164"/>
-      <c r="H1" s="158" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="158"/>
-      <c r="J1" s="159" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="159"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="156"/>
-      <c r="B2" s="156"/>
-      <c r="C2" s="157"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="157"/>
-      <c r="F2" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="153" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="153">
-        <v>1320</v>
-      </c>
-      <c r="D3" s="153" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="3">
-        <v>100</v>
-      </c>
-      <c r="F3" s="10">
-        <v>0.23</v>
-      </c>
-      <c r="G3" s="10">
-        <v>0.05</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="154"/>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="154"/>
-      <c r="D4" s="155"/>
-      <c r="E4" s="1">
-        <v>100</v>
-      </c>
-      <c r="F4" s="7">
-        <v>0.17</v>
-      </c>
-      <c r="G4" s="7">
-        <v>0.02</v>
-      </c>
-      <c r="H4" s="8">
-        <v>0.15</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0.19</v>
-      </c>
-      <c r="J4" s="9">
-        <v>0.67</v>
-      </c>
-      <c r="K4" s="9">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="154"/>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="154"/>
-      <c r="D5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="2">
-        <f>3.5*2</f>
-        <v>7</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0.41</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0.08</v>
-      </c>
-      <c r="H5" s="5">
-        <v>0.59</v>
-      </c>
-      <c r="I5" s="5">
-        <v>0.4</v>
-      </c>
-      <c r="J5" s="6">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="154"/>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="154"/>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="2">
-        <f>13.9*2</f>
-        <v>27.8</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0.16</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0.03</v>
-      </c>
-      <c r="H6" s="5">
-        <v>0.83</v>
-      </c>
-      <c r="I6" s="5">
-        <v>0.36</v>
-      </c>
-      <c r="J6" s="6">
-        <v>0</v>
-      </c>
-      <c r="K6" s="6">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="155"/>
-      <c r="B7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="155"/>
-      <c r="D7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="2">
-        <f>8.5*2</f>
-        <v>17</v>
-      </c>
-      <c r="F7" s="4">
-        <v>0.38</v>
-      </c>
-      <c r="G7" s="4">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="H7" s="5">
-        <v>0.62</v>
-      </c>
-      <c r="I7" s="5">
-        <v>0.39</v>
-      </c>
-      <c r="J7" s="6">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6">
-        <v>0.54</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
1, 2, 3 layers (1064, 1550nm)
Change SiO2 substrate dataset
</commit_message>
<xml_diff>
--- a/meetings/AsymReca_ThkCalc.xlsx
+++ b/meetings/AsymReca_ThkCalc.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2024-ILLUSTRIOUS\My Drive (61050734@kmitl.ac.th)\AsymReca_SbSe\meetings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2FC23C-293D-4400-8BE6-65195114BC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F4761F-2615-4F45-A2E6-345854E25F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28200" yWindow="5265" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="532" sheetId="8" r:id="rId1"/>
-    <sheet name="600" sheetId="10" r:id="rId2"/>
-    <sheet name="700" sheetId="11" r:id="rId3"/>
-    <sheet name="800" sheetId="12" r:id="rId4"/>
-    <sheet name="1064" sheetId="9" r:id="rId5"/>
-    <sheet name="Amorphous phase" sheetId="7" state="hidden" r:id="rId6"/>
-    <sheet name="1064_back" sheetId="13" r:id="rId7"/>
-    <sheet name="Crystalline" sheetId="4" r:id="rId8"/>
-    <sheet name="Sheet2" sheetId="5" state="hidden" r:id="rId9"/>
-    <sheet name="Sheet3" sheetId="6" state="hidden" r:id="rId10"/>
+    <sheet name="1064_back" sheetId="13" r:id="rId1"/>
+    <sheet name="1550_back" sheetId="14" r:id="rId2"/>
+    <sheet name="532" sheetId="8" r:id="rId3"/>
+    <sheet name="600" sheetId="10" r:id="rId4"/>
+    <sheet name="700" sheetId="11" r:id="rId5"/>
+    <sheet name="800" sheetId="12" r:id="rId6"/>
+    <sheet name="1064" sheetId="9" r:id="rId7"/>
+    <sheet name="Amorphous phase" sheetId="7" state="hidden" r:id="rId8"/>
+    <sheet name="Crystalline" sheetId="4" r:id="rId9"/>
+    <sheet name="Sheet2" sheetId="5" state="hidden" r:id="rId10"/>
+    <sheet name="Sheet3" sheetId="6" state="hidden" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="109">
   <si>
     <t>Wavelength (nm)</t>
   </si>
@@ -2297,7 +2298,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="170">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2666,22 +2667,46 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2690,6 +2715,12 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2697,30 +2728,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2729,12 +2736,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -2803,15 +2804,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2819,17 +2811,7 @@
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="51">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2847,46 +2829,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3012,6 +2954,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3027,6 +2999,316 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3315,6 +3597,1885 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6C66A9-86C5-4B44-B720-CA86E494EFA2}">
+  <dimension ref="A1:U28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" style="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="35" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" style="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" style="44" customWidth="1"/>
+    <col min="5" max="5" width="7.7109375" style="34" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" style="84" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" style="43" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" style="91" customWidth="1"/>
+    <col min="9" max="9" width="7.28515625" style="92" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" style="41" customWidth="1"/>
+    <col min="11" max="12" width="7.28515625" style="92" customWidth="1"/>
+    <col min="13" max="13" width="7.28515625" style="41" customWidth="1"/>
+    <col min="14" max="15" width="7.28515625" style="92" customWidth="1"/>
+    <col min="16" max="16" width="7.28515625" style="41" customWidth="1"/>
+    <col min="17" max="21" width="7.28515625" style="32" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="32"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="133" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="140" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="135" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="138" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="131"/>
+      <c r="J1" s="132"/>
+      <c r="K1" s="130" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
+        <v>3</v>
+      </c>
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+    </row>
+    <row r="2" spans="1:21" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="134"/>
+      <c r="B2" s="141"/>
+      <c r="C2" s="136"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="127"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="129"/>
+      <c r="H2" s="111" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="52" t="s">
+        <v>50</v>
+      </c>
+      <c r="N2" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="O2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="P2" s="52" t="s">
+        <v>51</v>
+      </c>
+      <c r="R2" s="127"/>
+      <c r="S2" s="127"/>
+      <c r="T2" s="127"/>
+      <c r="U2" s="127"/>
+    </row>
+    <row r="3" spans="1:21" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="30">
+        <v>1064</v>
+      </c>
+      <c r="B3" s="35"/>
+      <c r="C3" s="45" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="82">
+        <v>0</v>
+      </c>
+      <c r="E3" s="31">
+        <v>0</v>
+      </c>
+      <c r="F3" s="84">
+        <v>157.88</v>
+      </c>
+      <c r="G3" s="83">
+        <f>F3</f>
+        <v>157.88</v>
+      </c>
+      <c r="H3" s="95">
+        <v>0.93500000000000005</v>
+      </c>
+      <c r="I3" s="96">
+        <v>0.372</v>
+      </c>
+      <c r="J3" s="90">
+        <f t="shared" ref="J3:J7" si="0">H3-I3</f>
+        <v>0.56300000000000006</v>
+      </c>
+      <c r="K3" s="96">
+        <v>0</v>
+      </c>
+      <c r="L3" s="96">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="M3" s="90">
+        <f t="shared" ref="M3:M7" si="1">K3-L3</f>
+        <v>-1.2999999999999999E-2</v>
+      </c>
+      <c r="N3" s="96">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="O3" s="96">
+        <v>0.61499999999999999</v>
+      </c>
+      <c r="P3" s="90">
+        <f t="shared" ref="P3:P7" si="2">N3-O3</f>
+        <v>-0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C4" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="44">
+        <v>115.17</v>
+      </c>
+      <c r="E4" s="34">
+        <v>0</v>
+      </c>
+      <c r="F4" s="84">
+        <v>157.88</v>
+      </c>
+      <c r="G4" s="43">
+        <f>D4+F4</f>
+        <v>273.05</v>
+      </c>
+      <c r="H4" s="91">
+        <v>0.93300000000000005</v>
+      </c>
+      <c r="I4" s="92">
+        <v>0.76900000000000002</v>
+      </c>
+      <c r="J4" s="90">
+        <f t="shared" si="0"/>
+        <v>0.16400000000000003</v>
+      </c>
+      <c r="K4" s="92">
+        <v>0</v>
+      </c>
+      <c r="L4" s="92">
+        <v>0.01</v>
+      </c>
+      <c r="M4" s="90">
+        <f t="shared" si="1"/>
+        <v>-0.01</v>
+      </c>
+      <c r="N4" s="92">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="O4" s="92">
+        <v>0.221</v>
+      </c>
+      <c r="P4" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.154</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B5" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="126">
+        <v>162.07</v>
+      </c>
+      <c r="E5" s="34">
+        <v>0</v>
+      </c>
+      <c r="F5" s="84">
+        <v>32.880000000000003</v>
+      </c>
+      <c r="G5" s="43">
+        <f>D5+F5</f>
+        <v>194.95</v>
+      </c>
+      <c r="H5" s="91">
+        <v>0.96599999999999997</v>
+      </c>
+      <c r="I5" s="92">
+        <v>0.82799999999999996</v>
+      </c>
+      <c r="J5" s="90">
+        <f>H5-I5</f>
+        <v>0.13800000000000001</v>
+      </c>
+      <c r="K5" s="92">
+        <v>0</v>
+      </c>
+      <c r="L5" s="92">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="M5" s="90">
+        <f>K5-L5</f>
+        <v>-8.0000000000000004E-4</v>
+      </c>
+      <c r="N5" s="92">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="O5" s="92">
+        <v>0.16400000000000001</v>
+      </c>
+      <c r="P5" s="90">
+        <f>N5-O5</f>
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B6" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="126">
+        <v>125</v>
+      </c>
+      <c r="E6" s="34">
+        <v>0</v>
+      </c>
+      <c r="F6" s="84">
+        <v>68.260000000000005</v>
+      </c>
+      <c r="G6" s="43">
+        <f>D6+F6</f>
+        <v>193.26</v>
+      </c>
+      <c r="H6" s="91">
+        <v>0.93600000000000005</v>
+      </c>
+      <c r="I6" s="92">
+        <v>0.73799999999999999</v>
+      </c>
+      <c r="J6" s="90">
+        <f t="shared" si="0"/>
+        <v>0.19800000000000006</v>
+      </c>
+      <c r="K6" s="92">
+        <v>0</v>
+      </c>
+      <c r="L6" s="92">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="M6" s="90">
+        <f t="shared" si="1"/>
+        <v>-8.9999999999999993E-3</v>
+      </c>
+      <c r="N6" s="92">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="O6" s="92">
+        <v>0.252</v>
+      </c>
+      <c r="P6" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C7" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="44">
+        <v>149.63999999999999</v>
+      </c>
+      <c r="E7" s="34">
+        <v>115.17</v>
+      </c>
+      <c r="F7" s="84">
+        <v>78.94</v>
+      </c>
+      <c r="G7" s="43">
+        <f>SUM(D7:F7)</f>
+        <v>343.75</v>
+      </c>
+      <c r="H7" s="91">
+        <v>0.93500000000000005</v>
+      </c>
+      <c r="I7" s="92">
+        <v>0.76900000000000002</v>
+      </c>
+      <c r="J7" s="90">
+        <f t="shared" si="0"/>
+        <v>0.16600000000000004</v>
+      </c>
+      <c r="K7" s="92">
+        <v>0</v>
+      </c>
+      <c r="L7" s="92">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="M7" s="90">
+        <f t="shared" si="1"/>
+        <v>-1.0999999999999999E-2</v>
+      </c>
+      <c r="N7" s="92">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="O7" s="92">
+        <v>0.221</v>
+      </c>
+      <c r="P7" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A8" s="30"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B9" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="44">
+        <v>181.31</v>
+      </c>
+      <c r="E9" s="34">
+        <v>193.08</v>
+      </c>
+      <c r="F9" s="84">
+        <v>157.88</v>
+      </c>
+      <c r="G9" s="43">
+        <f>SUM(D9:F9)</f>
+        <v>532.27</v>
+      </c>
+      <c r="H9" s="91">
+        <v>0.95</v>
+      </c>
+      <c r="I9" s="92">
+        <v>0.55800000000000005</v>
+      </c>
+      <c r="J9" s="90">
+        <f>H9-I9</f>
+        <v>0.3919999999999999</v>
+      </c>
+      <c r="K9" s="92">
+        <v>0</v>
+      </c>
+      <c r="L9" s="92">
+        <v>1.9E-2</v>
+      </c>
+      <c r="M9" s="90">
+        <f>K9-L9</f>
+        <v>-1.9E-2</v>
+      </c>
+      <c r="N9" s="92">
+        <v>0.05</v>
+      </c>
+      <c r="O9" s="92">
+        <v>0.42299999999999999</v>
+      </c>
+      <c r="P9" s="90">
+        <f>N9-O9</f>
+        <v>-0.373</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A10" s="30"/>
+      <c r="B10" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="D10" s="44">
+        <v>164.55</v>
+      </c>
+      <c r="E10" s="34">
+        <v>193.08</v>
+      </c>
+      <c r="F10" s="84">
+        <f>F9</f>
+        <v>157.88</v>
+      </c>
+      <c r="G10" s="43">
+        <f>SUM(D10:F10)</f>
+        <v>515.51</v>
+      </c>
+      <c r="H10" s="91">
+        <v>0.96599999999999997</v>
+      </c>
+      <c r="I10" s="92">
+        <v>0.627</v>
+      </c>
+      <c r="J10" s="90">
+        <f>H10-I10</f>
+        <v>0.33899999999999997</v>
+      </c>
+      <c r="K10" s="92">
+        <v>0</v>
+      </c>
+      <c r="L10" s="92">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="M10" s="90">
+        <f>K10-L10</f>
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="N10" s="92">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="O10" s="92">
+        <v>0.35399999999999998</v>
+      </c>
+      <c r="P10" s="90">
+        <f>N10-O10</f>
+        <v>-0.31999999999999995</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B11" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" s="44">
+        <v>133.22999999999999</v>
+      </c>
+      <c r="E11" s="34">
+        <v>164.55</v>
+      </c>
+      <c r="F11" s="84">
+        <f t="shared" ref="F11:F12" si="3">F10</f>
+        <v>157.88</v>
+      </c>
+      <c r="G11" s="43">
+        <f>SUM(D11:F11)</f>
+        <v>455.65999999999997</v>
+      </c>
+      <c r="H11" s="91">
+        <v>0.96599999999999997</v>
+      </c>
+      <c r="I11" s="92">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="J11" s="90">
+        <f>H11-I11</f>
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="K11" s="92">
+        <v>0</v>
+      </c>
+      <c r="L11" s="92">
+        <v>1.9E-2</v>
+      </c>
+      <c r="M11" s="90">
+        <f>K11-L11</f>
+        <v>-1.9E-2</v>
+      </c>
+      <c r="N11" s="92">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="O11" s="92">
+        <v>0.14799999999999999</v>
+      </c>
+      <c r="P11" s="90">
+        <f>N11-O11</f>
+        <v>-0.11399999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B12" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="44">
+        <v>115.17</v>
+      </c>
+      <c r="E12" s="34">
+        <v>133.22999999999999</v>
+      </c>
+      <c r="F12" s="84">
+        <f t="shared" si="3"/>
+        <v>157.88</v>
+      </c>
+      <c r="G12" s="43">
+        <f>SUM(D12:F12)</f>
+        <v>406.28</v>
+      </c>
+      <c r="H12" s="91">
+        <v>0.96499999999999997</v>
+      </c>
+      <c r="I12" s="92">
+        <v>0.94099999999999995</v>
+      </c>
+      <c r="J12" s="90">
+        <f>H12-I12</f>
+        <v>2.4000000000000021E-2</v>
+      </c>
+      <c r="K12" s="92">
+        <v>0</v>
+      </c>
+      <c r="L12" s="92">
+        <v>1.9E-2</v>
+      </c>
+      <c r="M12" s="90">
+        <f>K12-L12</f>
+        <v>-1.9E-2</v>
+      </c>
+      <c r="N12" s="92">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="O12" s="92">
+        <v>0.04</v>
+      </c>
+      <c r="P12" s="90">
+        <f>N12-O12</f>
+        <v>-4.9999999999999975E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B18" s="71"/>
+      <c r="J18" s="97"/>
+      <c r="M18" s="97"/>
+      <c r="P18" s="97"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="71"/>
+      <c r="J19" s="97"/>
+      <c r="M19" s="97"/>
+      <c r="P19" s="97"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J20" s="97"/>
+      <c r="M20" s="97"/>
+      <c r="P20" s="97"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J21" s="97"/>
+      <c r="M21" s="97"/>
+      <c r="P21" s="97"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="C23" s="37"/>
+      <c r="D23" s="122"/>
+      <c r="J23" s="97"/>
+      <c r="M23" s="97"/>
+      <c r="P23" s="97"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="30"/>
+      <c r="D24" s="122"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="D25" s="122"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="30"/>
+      <c r="C26" s="37"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="30"/>
+      <c r="C27" s="118"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J15:J1048576 J1:J12">
+    <cfRule type="top10" dxfId="16" priority="1" percent="1" rank="25"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BF2213B-BB65-498C-AA64-42693820505C}">
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" style="17" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" style="17" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" style="17" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="17" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="A1" s="169" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="169" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="164" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="164" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="164" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="165" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="165"/>
+      <c r="H1" s="158" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="158"/>
+      <c r="J1" s="159" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="159"/>
+    </row>
+    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2" s="169"/>
+      <c r="B2" s="169"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="160" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="160">
+        <v>1550</v>
+      </c>
+      <c r="D3" s="160" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="13">
+        <v>52</v>
+      </c>
+      <c r="F3" s="14">
+        <v>0.48</v>
+      </c>
+      <c r="G3" s="14">
+        <v>0.16</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="161"/>
+      <c r="B4" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="161"/>
+      <c r="D4" s="163"/>
+      <c r="E4" s="18">
+        <v>52</v>
+      </c>
+      <c r="F4" s="27">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="G4" s="27">
+        <v>0.11</v>
+      </c>
+      <c r="H4" s="28">
+        <v>0.44</v>
+      </c>
+      <c r="I4" s="28">
+        <v>0.38</v>
+      </c>
+      <c r="J4" s="29">
+        <v>0</v>
+      </c>
+      <c r="K4" s="29">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="161"/>
+      <c r="B5" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="161"/>
+      <c r="D5" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="19">
+        <f>2.6*2</f>
+        <v>5.2</v>
+      </c>
+      <c r="F5" s="20">
+        <v>0.41</v>
+      </c>
+      <c r="G5" s="20">
+        <v>0.04</v>
+      </c>
+      <c r="H5" s="21">
+        <v>0.59</v>
+      </c>
+      <c r="I5" s="21">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="J5" s="22">
+        <v>0</v>
+      </c>
+      <c r="K5" s="22">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="162"/>
+      <c r="B6" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="162"/>
+      <c r="D6" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="23">
+        <f>6.6*2</f>
+        <v>13.2</v>
+      </c>
+      <c r="F6" s="24">
+        <v>0.41</v>
+      </c>
+      <c r="G6" s="24">
+        <v>0.04</v>
+      </c>
+      <c r="H6" s="25">
+        <v>0.59</v>
+      </c>
+      <c r="I6" s="25">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="J6" s="26">
+        <v>0</v>
+      </c>
+      <c r="K6" s="26">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="166" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="166">
+        <v>1320</v>
+      </c>
+      <c r="D7" s="166" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="3">
+        <v>100</v>
+      </c>
+      <c r="F7" s="10">
+        <v>0.23</v>
+      </c>
+      <c r="G7" s="10">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="167"/>
+      <c r="B8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="167"/>
+      <c r="D8" s="168"/>
+      <c r="E8" s="1">
+        <v>100</v>
+      </c>
+      <c r="F8" s="7">
+        <v>0.17</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="H8" s="8">
+        <v>0.15</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0.19</v>
+      </c>
+      <c r="J8" s="9">
+        <v>0.67</v>
+      </c>
+      <c r="K8" s="9">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="167"/>
+      <c r="B9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="167"/>
+      <c r="D9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="2">
+        <f>3.5*2</f>
+        <v>7</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0.41</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0.08</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0.59</v>
+      </c>
+      <c r="I9" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="J9" s="6">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="167"/>
+      <c r="B10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="167"/>
+      <c r="D10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="2">
+        <f>13.9*2</f>
+        <v>27.8</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="H10" s="5">
+        <v>0.83</v>
+      </c>
+      <c r="I10" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="J10" s="6">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="168"/>
+      <c r="B11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="168"/>
+      <c r="D11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="2">
+        <f>8.5*2</f>
+        <v>17</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0.38</v>
+      </c>
+      <c r="G11" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="H11" s="5">
+        <v>0.62</v>
+      </c>
+      <c r="I11" s="5">
+        <v>0.39</v>
+      </c>
+      <c r="J11" s="6">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6">
+        <v>0.54</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37079731-60AB-4D94-B991-690660612702}">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="169" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="169" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="164" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="164" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="164" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="165" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="165"/>
+      <c r="H1" s="158" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="158"/>
+      <c r="J1" s="159" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="159"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="169"/>
+      <c r="B2" s="169"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="166" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="166">
+        <v>1320</v>
+      </c>
+      <c r="D3" s="166" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="3">
+        <v>100</v>
+      </c>
+      <c r="F3" s="10">
+        <v>0.23</v>
+      </c>
+      <c r="G3" s="10">
+        <v>0.05</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="167"/>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="167"/>
+      <c r="D4" s="168"/>
+      <c r="E4" s="1">
+        <v>100</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0.17</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="H4" s="8">
+        <v>0.15</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0.19</v>
+      </c>
+      <c r="J4" s="9">
+        <v>0.67</v>
+      </c>
+      <c r="K4" s="9">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="167"/>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="167"/>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="2">
+        <f>3.5*2</f>
+        <v>7</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.41</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0.08</v>
+      </c>
+      <c r="H5" s="5">
+        <v>0.59</v>
+      </c>
+      <c r="I5" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="167"/>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="167"/>
+      <c r="D6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="2">
+        <f>13.9*2</f>
+        <v>27.8</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="H6" s="5">
+        <v>0.83</v>
+      </c>
+      <c r="I6" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="168"/>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="168"/>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2">
+        <f>8.5*2</f>
+        <v>17</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.38</v>
+      </c>
+      <c r="G7" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0.62</v>
+      </c>
+      <c r="I7" s="5">
+        <v>0.39</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0.54</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7F0F96A-322F-4AD3-A595-EC2EEF5FB330}">
+  <dimension ref="A1:U28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" style="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="35" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" style="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" style="44" customWidth="1"/>
+    <col min="5" max="5" width="7.7109375" style="34" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" style="84" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" style="43" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" style="91" customWidth="1"/>
+    <col min="9" max="9" width="7.28515625" style="92" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" style="41" customWidth="1"/>
+    <col min="11" max="12" width="7.28515625" style="92" customWidth="1"/>
+    <col min="13" max="13" width="7.28515625" style="41" customWidth="1"/>
+    <col min="14" max="15" width="7.28515625" style="92" customWidth="1"/>
+    <col min="16" max="16" width="7.28515625" style="41" customWidth="1"/>
+    <col min="17" max="21" width="7.28515625" style="32" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="32"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="133" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="140" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="135" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="138" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="131"/>
+      <c r="J1" s="132"/>
+      <c r="K1" s="130" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
+        <v>3</v>
+      </c>
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+    </row>
+    <row r="2" spans="1:21" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="134"/>
+      <c r="B2" s="141"/>
+      <c r="C2" s="136"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="127"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="129"/>
+      <c r="H2" s="111" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="52" t="s">
+        <v>50</v>
+      </c>
+      <c r="N2" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="O2" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="P2" s="52" t="s">
+        <v>51</v>
+      </c>
+      <c r="R2" s="127"/>
+      <c r="S2" s="127"/>
+      <c r="T2" s="127"/>
+      <c r="U2" s="127"/>
+    </row>
+    <row r="3" spans="1:21" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="30">
+        <v>1064</v>
+      </c>
+      <c r="B3" s="35"/>
+      <c r="C3" s="45" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="82">
+        <v>0</v>
+      </c>
+      <c r="E3" s="31">
+        <v>0</v>
+      </c>
+      <c r="F3" s="84">
+        <v>235.89</v>
+      </c>
+      <c r="G3" s="83">
+        <f>F3</f>
+        <v>235.89</v>
+      </c>
+      <c r="H3" s="95">
+        <v>0.93600000000000005</v>
+      </c>
+      <c r="I3" s="96">
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="J3" s="90">
+        <f t="shared" ref="J3:J7" si="0">H3-I3</f>
+        <v>0.46100000000000008</v>
+      </c>
+      <c r="K3" s="96">
+        <v>0</v>
+      </c>
+      <c r="L3" s="96">
+        <v>0</v>
+      </c>
+      <c r="M3" s="90">
+        <f t="shared" ref="M3:M7" si="1">K3-L3</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="96">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="O3" s="96">
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="P3" s="90">
+        <f t="shared" ref="P3:P7" si="2">N3-O3</f>
+        <v>-0.46100000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C4" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="44">
+        <v>169.22</v>
+      </c>
+      <c r="E4" s="34">
+        <v>0</v>
+      </c>
+      <c r="F4" s="84">
+        <v>117.95</v>
+      </c>
+      <c r="G4" s="43">
+        <f>D4+F4</f>
+        <v>287.17</v>
+      </c>
+      <c r="H4" s="91">
+        <v>0.93799999999999994</v>
+      </c>
+      <c r="I4" s="92">
+        <v>0.81200000000000006</v>
+      </c>
+      <c r="J4" s="90">
+        <f t="shared" si="0"/>
+        <v>0.12599999999999989</v>
+      </c>
+      <c r="K4" s="92">
+        <v>0</v>
+      </c>
+      <c r="L4" s="92">
+        <v>0</v>
+      </c>
+      <c r="M4" s="90">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N4" s="92">
+        <v>6.2E-2</v>
+      </c>
+      <c r="O4" s="92">
+        <v>0.188</v>
+      </c>
+      <c r="P4" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B5" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="44">
+        <v>239.9</v>
+      </c>
+      <c r="E5" s="34">
+        <v>0</v>
+      </c>
+      <c r="F5" s="84">
+        <v>47.41</v>
+      </c>
+      <c r="G5" s="43">
+        <f>D5+F5</f>
+        <v>287.31</v>
+      </c>
+      <c r="H5" s="91">
+        <v>0.96699999999999997</v>
+      </c>
+      <c r="I5" s="92">
+        <v>0.88800000000000001</v>
+      </c>
+      <c r="J5" s="90">
+        <f t="shared" si="0"/>
+        <v>7.8999999999999959E-2</v>
+      </c>
+      <c r="K5" s="92">
+        <v>0</v>
+      </c>
+      <c r="L5" s="92">
+        <v>0</v>
+      </c>
+      <c r="M5" s="90">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N5" s="92">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="O5" s="92">
+        <v>0.112</v>
+      </c>
+      <c r="P5" s="90">
+        <f t="shared" si="2"/>
+        <v>-7.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B6" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="126">
+        <v>98.51</v>
+      </c>
+      <c r="E6" s="34">
+        <v>0</v>
+      </c>
+      <c r="F6" s="84">
+        <v>185.42</v>
+      </c>
+      <c r="G6" s="43">
+        <f>D6+F6</f>
+        <v>283.93</v>
+      </c>
+      <c r="H6" s="91">
+        <v>0.96699999999999997</v>
+      </c>
+      <c r="I6" s="92">
+        <v>0.80200000000000005</v>
+      </c>
+      <c r="J6" s="90">
+        <f t="shared" si="0"/>
+        <v>0.16499999999999992</v>
+      </c>
+      <c r="K6" s="92">
+        <v>0</v>
+      </c>
+      <c r="L6" s="92">
+        <v>0</v>
+      </c>
+      <c r="M6" s="90">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N6" s="92">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="O6" s="92">
+        <v>0.19700000000000001</v>
+      </c>
+      <c r="P6" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.16400000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C7" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="44">
+        <v>222.73</v>
+      </c>
+      <c r="E7" s="34">
+        <v>169.22</v>
+      </c>
+      <c r="F7" s="84">
+        <v>117.95</v>
+      </c>
+      <c r="G7" s="43">
+        <f>SUM(D7:F7)</f>
+        <v>509.9</v>
+      </c>
+      <c r="H7" s="91">
+        <v>0.93799999999999994</v>
+      </c>
+      <c r="I7" s="92">
+        <v>0.81100000000000005</v>
+      </c>
+      <c r="J7" s="90">
+        <f t="shared" si="0"/>
+        <v>0.12699999999999989</v>
+      </c>
+      <c r="K7" s="92">
+        <v>0</v>
+      </c>
+      <c r="L7" s="92">
+        <v>0</v>
+      </c>
+      <c r="M7" s="90">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N7" s="92">
+        <v>6.2E-2</v>
+      </c>
+      <c r="O7" s="92">
+        <v>0.188</v>
+      </c>
+      <c r="P7" s="90">
+        <f t="shared" si="2"/>
+        <v>-0.126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A8" s="30"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B9" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="44">
+        <v>268.3</v>
+      </c>
+      <c r="E9" s="34">
+        <v>281.89999999999998</v>
+      </c>
+      <c r="F9" s="84">
+        <v>235.89</v>
+      </c>
+      <c r="G9" s="43">
+        <f>SUM(D9:F9)</f>
+        <v>786.09</v>
+      </c>
+      <c r="H9" s="91">
+        <v>0.95</v>
+      </c>
+      <c r="I9" s="92">
+        <v>0.66200000000000003</v>
+      </c>
+      <c r="J9" s="90">
+        <f>H9-I9</f>
+        <v>0.28799999999999992</v>
+      </c>
+      <c r="K9" s="92">
+        <v>0</v>
+      </c>
+      <c r="L9" s="92">
+        <v>1E-3</v>
+      </c>
+      <c r="M9" s="90">
+        <f>K9-L9</f>
+        <v>-1E-3</v>
+      </c>
+      <c r="N9" s="92">
+        <v>0.05</v>
+      </c>
+      <c r="O9" s="92">
+        <v>0.33800000000000002</v>
+      </c>
+      <c r="P9" s="90">
+        <f>N9-O9</f>
+        <v>-0.28800000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A10" s="30"/>
+      <c r="B10" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="D10" s="44">
+        <v>240.07</v>
+      </c>
+      <c r="E10" s="34">
+        <v>281.89999999999998</v>
+      </c>
+      <c r="F10" s="84">
+        <v>235.89</v>
+      </c>
+      <c r="G10" s="43">
+        <f>SUM(D10:F10)</f>
+        <v>757.86</v>
+      </c>
+      <c r="H10" s="91">
+        <v>0.96599999999999997</v>
+      </c>
+      <c r="I10" s="92">
+        <v>0.72899999999999998</v>
+      </c>
+      <c r="J10" s="90">
+        <f>H10-I10</f>
+        <v>0.23699999999999999</v>
+      </c>
+      <c r="K10" s="92">
+        <v>0</v>
+      </c>
+      <c r="L10" s="92">
+        <v>0</v>
+      </c>
+      <c r="M10" s="90">
+        <f>K10-L10</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="92">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="O10" s="92">
+        <v>0.27100000000000002</v>
+      </c>
+      <c r="P10" s="90">
+        <f>N10-O10</f>
+        <v>-0.23700000000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B11" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" s="44">
+        <v>194.68</v>
+      </c>
+      <c r="E11" s="34">
+        <v>240.07</v>
+      </c>
+      <c r="F11" s="84">
+        <v>235.89</v>
+      </c>
+      <c r="G11" s="43">
+        <f>SUM(D11:F11)</f>
+        <v>670.64</v>
+      </c>
+      <c r="H11" s="91">
+        <v>0.96599999999999997</v>
+      </c>
+      <c r="I11" s="92">
+        <v>0.89600000000000002</v>
+      </c>
+      <c r="J11" s="90">
+        <f>H11-I11</f>
+        <v>6.9999999999999951E-2</v>
+      </c>
+      <c r="K11" s="92">
+        <v>0</v>
+      </c>
+      <c r="L11" s="92">
+        <v>0</v>
+      </c>
+      <c r="M11" s="90">
+        <f>K11-L11</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="92">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="O11" s="92">
+        <v>0.104</v>
+      </c>
+      <c r="P11" s="90">
+        <f>N11-O11</f>
+        <v>-6.9999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B12" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="44">
+        <v>169.22</v>
+      </c>
+      <c r="E12" s="34">
+        <v>194.68</v>
+      </c>
+      <c r="F12" s="84">
+        <v>235.89</v>
+      </c>
+      <c r="G12" s="43">
+        <f>SUM(D12:F12)</f>
+        <v>599.79</v>
+      </c>
+      <c r="H12" s="91">
+        <v>0.96499999999999997</v>
+      </c>
+      <c r="I12" s="92">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="J12" s="90">
+        <f>H12-I12</f>
+        <v>1.0000000000000009E-3</v>
+      </c>
+      <c r="K12" s="92">
+        <v>0</v>
+      </c>
+      <c r="L12" s="92">
+        <v>0</v>
+      </c>
+      <c r="M12" s="90">
+        <f>K12-L12</f>
+        <v>0</v>
+      </c>
+      <c r="N12" s="92">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="O12" s="92">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="P12" s="90">
+        <f>N12-O12</f>
+        <v>-9.9999999999999395E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B18" s="71"/>
+      <c r="J18" s="97"/>
+      <c r="M18" s="97"/>
+      <c r="P18" s="97"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="71"/>
+      <c r="J19" s="97"/>
+      <c r="M19" s="97"/>
+      <c r="P19" s="97"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J20" s="97"/>
+      <c r="M20" s="97"/>
+      <c r="P20" s="97"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J21" s="97"/>
+      <c r="M21" s="97"/>
+      <c r="P21" s="97"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="C23" s="37"/>
+      <c r="D23" s="122"/>
+      <c r="J23" s="97"/>
+      <c r="M23" s="97"/>
+      <c r="P23" s="97"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="30"/>
+      <c r="D24" s="122"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="D25" s="122"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="30"/>
+      <c r="C26" s="37"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="30"/>
+      <c r="C27" s="118"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="R2:S2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J15:J1048576 J1:J12">
+    <cfRule type="top10" dxfId="15" priority="1" percent="1" rank="25"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{983CE563-D765-4D88-816D-AF600C9A68D9}">
   <dimension ref="A1:Y42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3342,65 +5503,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="133" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="139" t="s">
+      <c r="C1" s="135" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="137" t="s">
+      <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="134" t="s">
+      <c r="F1" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="130" t="s">
+      <c r="G1" s="138" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="132" t="s">
+      <c r="H1" s="142" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="134" t="s">
+      <c r="I1" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="135" t="s">
+      <c r="J1" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="137" t="s">
+      <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="134"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="137" t="s">
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="134"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="137" t="s">
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+      <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="134"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="127" t="s">
+      <c r="R1" s="131"/>
+      <c r="S1" s="132"/>
+      <c r="T1" s="133" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128"/>
+      <c r="A2" s="134"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="140"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="131"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="136"/>
+      <c r="C2" s="136"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="129"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -3428,11 +5589,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="128"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
+      <c r="T2" s="134"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -4715,23 +6876,8 @@
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:P1"/>
   </mergeCells>
-  <conditionalFormatting sqref="M4:M18">
-    <cfRule type="cellIs" dxfId="21" priority="2" operator="greaterThan">
-      <formula>$M$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M20:M21">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
-      <formula>$M$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M40:M42">
-    <cfRule type="cellIs" dxfId="19" priority="4" operator="greaterThan">
-      <formula>0.45</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="greaterThan">
-      <formula>0.45</formula>
-    </cfRule>
+  <conditionalFormatting sqref="M1:M1048576">
+    <cfRule type="top10" dxfId="14" priority="1" percent="1" rank="25"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A20" r:id="rId1" xr:uid="{0CA2BC15-2917-4413-A3B6-CA9BB1B2A39C}"/>
@@ -4740,251 +6886,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37079731-60AB-4D94-B991-690660612702}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="169" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="169" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="164" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="164" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="164" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="165" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="165"/>
-      <c r="H1" s="158" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="158"/>
-      <c r="J1" s="159" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="159"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="169"/>
-      <c r="B2" s="169"/>
-      <c r="C2" s="164"/>
-      <c r="D2" s="164"/>
-      <c r="E2" s="164"/>
-      <c r="F2" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="166" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="166">
-        <v>1320</v>
-      </c>
-      <c r="D3" s="166" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="3">
-        <v>100</v>
-      </c>
-      <c r="F3" s="10">
-        <v>0.23</v>
-      </c>
-      <c r="G3" s="10">
-        <v>0.05</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="167"/>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="167"/>
-      <c r="D4" s="168"/>
-      <c r="E4" s="1">
-        <v>100</v>
-      </c>
-      <c r="F4" s="7">
-        <v>0.17</v>
-      </c>
-      <c r="G4" s="7">
-        <v>0.02</v>
-      </c>
-      <c r="H4" s="8">
-        <v>0.15</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0.19</v>
-      </c>
-      <c r="J4" s="9">
-        <v>0.67</v>
-      </c>
-      <c r="K4" s="9">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="167"/>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="167"/>
-      <c r="D5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="2">
-        <f>3.5*2</f>
-        <v>7</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0.41</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0.08</v>
-      </c>
-      <c r="H5" s="5">
-        <v>0.59</v>
-      </c>
-      <c r="I5" s="5">
-        <v>0.4</v>
-      </c>
-      <c r="J5" s="6">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="167"/>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="167"/>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="2">
-        <f>13.9*2</f>
-        <v>27.8</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0.16</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0.03</v>
-      </c>
-      <c r="H6" s="5">
-        <v>0.83</v>
-      </c>
-      <c r="I6" s="5">
-        <v>0.36</v>
-      </c>
-      <c r="J6" s="6">
-        <v>0</v>
-      </c>
-      <c r="K6" s="6">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="168"/>
-      <c r="B7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="168"/>
-      <c r="D7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="2">
-        <f>8.5*2</f>
-        <v>17</v>
-      </c>
-      <c r="F7" s="4">
-        <v>0.38</v>
-      </c>
-      <c r="G7" s="4">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="H7" s="5">
-        <v>0.62</v>
-      </c>
-      <c r="I7" s="5">
-        <v>0.39</v>
-      </c>
-      <c r="J7" s="6">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6">
-        <v>0.54</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C52FA96-3BF9-4079-BB84-B7E23DF33659}">
   <dimension ref="A1:Y25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5012,65 +6914,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="133" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="143" t="s">
+      <c r="C1" s="145" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="137" t="s">
+      <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="134" t="s">
+      <c r="F1" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="130" t="s">
+      <c r="G1" s="138" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="142" t="s">
+      <c r="H1" s="144" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="134" t="s">
+      <c r="I1" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="135" t="s">
+      <c r="J1" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="137" t="s">
+      <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="134"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="137" t="s">
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="134"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="137" t="s">
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+      <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="134"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="127" t="s">
+      <c r="R1" s="131"/>
+      <c r="S1" s="132"/>
+      <c r="T1" s="133" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128"/>
+      <c r="A2" s="134"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="144"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="131"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="136"/>
+      <c r="C2" s="146"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="129"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -5098,11 +7000,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="128"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
+      <c r="T2" s="134"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -6042,12 +7944,12 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M4:M17">
-    <cfRule type="cellIs" dxfId="18" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -6058,7 +7960,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6885B2BD-93DD-45DD-89C8-7A5E1FBCD2B4}">
   <dimension ref="A1:Y25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6086,65 +7988,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="133" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="143" t="s">
+      <c r="C1" s="145" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="137" t="s">
+      <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="134" t="s">
+      <c r="F1" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="130" t="s">
+      <c r="G1" s="138" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="142" t="s">
+      <c r="H1" s="144" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="134" t="s">
+      <c r="I1" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="135" t="s">
+      <c r="J1" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="137" t="s">
+      <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="134"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="137" t="s">
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="134"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="137" t="s">
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+      <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="134"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="127" t="s">
+      <c r="R1" s="131"/>
+      <c r="S1" s="132"/>
+      <c r="T1" s="133" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128"/>
+      <c r="A2" s="134"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="144"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="131"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="136"/>
+      <c r="C2" s="146"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="129"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -6172,11 +8074,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="128"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
+      <c r="T2" s="134"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -6856,12 +8758,12 @@
     <mergeCell ref="T1:T2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M12">
-    <cfRule type="cellIs" dxfId="16" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="15" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -6872,7 +8774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9EC3644-111D-4FC3-90B7-D98EA9993FEE}">
   <dimension ref="A1:Y25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6900,65 +8802,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="133" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="143" t="s">
+      <c r="C1" s="145" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="137" t="s">
+      <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="134" t="s">
+      <c r="F1" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="130" t="s">
+      <c r="G1" s="138" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="142" t="s">
+      <c r="H1" s="144" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="134" t="s">
+      <c r="I1" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="135" t="s">
+      <c r="J1" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="137" t="s">
+      <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="134"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="137" t="s">
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="134"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="137" t="s">
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+      <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="134"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="127" t="s">
+      <c r="R1" s="131"/>
+      <c r="S1" s="132"/>
+      <c r="T1" s="133" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128"/>
+      <c r="A2" s="134"/>
       <c r="B2" s="115"/>
-      <c r="C2" s="144"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="131"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="136"/>
+      <c r="C2" s="146"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="129"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -6986,11 +8888,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="128"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
+      <c r="T2" s="134"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
@@ -7549,12 +9451,12 @@
     <mergeCell ref="G1:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M7 M10:M11">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23:M25">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -7565,7 +9467,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C373C9F4-FBF0-43BC-93B8-9C26388C4D3B}">
   <dimension ref="A1:Y30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7593,65 +9495,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="133" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="139" t="s">
+      <c r="C1" s="135" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="137" t="s">
+      <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="134" t="s">
+      <c r="F1" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="130" t="s">
+      <c r="G1" s="138" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="132" t="s">
+      <c r="H1" s="142" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="134" t="s">
+      <c r="I1" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="135" t="s">
+      <c r="J1" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="137" t="s">
+      <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="134"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="137" t="s">
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="134"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="137" t="s">
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+      <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="134"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="145" t="s">
+      <c r="R1" s="131"/>
+      <c r="S1" s="132"/>
+      <c r="T1" s="140" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128"/>
+      <c r="A2" s="134"/>
       <c r="B2" s="86"/>
-      <c r="C2" s="140"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="131"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="136"/>
+      <c r="C2" s="136"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="129"/>
       <c r="K2" s="111" t="s">
         <v>36</v>
       </c>
@@ -7679,11 +9581,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="146"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
+      <c r="T2" s="141"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
@@ -7798,7 +9700,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="P4" s="97">
-        <f t="shared" ref="P3:P6" si="2">N4-O4</f>
+        <f t="shared" ref="P4:P6" si="2">N4-O4</f>
         <v>-1.5000000000000444E-2</v>
       </c>
       <c r="Q4" s="92">
@@ -8555,7 +10457,7 @@
         <f>R19-Q19</f>
         <v>-0.48499999999999999</v>
       </c>
-      <c r="T19" s="126" t="s">
+      <c r="T19" s="125" t="s">
         <v>107</v>
       </c>
     </row>
@@ -8746,7 +10648,7 @@
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="C23" s="125"/>
+      <c r="C23" s="124"/>
       <c r="M23" s="97"/>
       <c r="P23" s="97"/>
       <c r="S23" s="97"/>
@@ -8939,12 +10841,12 @@
     <mergeCell ref="T1:T2"/>
   </mergeCells>
   <conditionalFormatting sqref="M4:M17 M19">
-    <cfRule type="cellIs" dxfId="12" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M16:M18">
-    <cfRule type="cellIs" dxfId="11" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="7" operator="greaterThan">
@@ -8952,17 +10854,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M20:M23">
-    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
       <formula>$M$19</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M25">
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="greaterThan">
-      <formula>$M$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M24">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="M24:M25">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>$M$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8970,7 +10867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2269C464-6090-4ACA-A164-907377F1E985}">
   <dimension ref="A1:Y33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9001,63 +10898,63 @@
       <c r="A1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="127" t="s">
+      <c r="B1" s="133" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="152" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="139" t="s">
+      <c r="D1" s="135" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="137" t="s">
+      <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="134" t="s">
+      <c r="F1" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="142" t="s">
+      <c r="G1" s="144" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="142" t="s">
+      <c r="H1" s="144" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="134" t="s">
+      <c r="I1" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="135" t="s">
+      <c r="J1" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="137" t="s">
+      <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="134"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="137" t="s">
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="134"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="137" t="s">
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+      <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="134"/>
-      <c r="S1" s="138"/>
+      <c r="R1" s="131"/>
+      <c r="S1" s="132"/>
       <c r="T1" s="151" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="129"/>
-      <c r="B2" s="128"/>
-      <c r="C2" s="144"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="136"/>
+      <c r="A2" s="127"/>
+      <c r="B2" s="134"/>
+      <c r="C2" s="146"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="134"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="129"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -9085,11 +10982,11 @@
       <c r="S2" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="129"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
+      <c r="T2" s="127"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="46">
@@ -10106,12 +12003,12 @@
     <mergeCell ref="G14:H14"/>
   </mergeCells>
   <conditionalFormatting sqref="M14:M20">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
       <formula>$M$13</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M29:M33">
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -10122,661 +12019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6C66A9-86C5-4B44-B720-CA86E494EFA2}">
-  <dimension ref="A1:W28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18.28515625" style="32" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" style="35" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" style="38" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" style="38" customWidth="1"/>
-    <col min="5" max="5" width="7.7109375" style="108" customWidth="1"/>
-    <col min="6" max="6" width="7.7109375" style="44" customWidth="1"/>
-    <col min="7" max="7" width="7.7109375" style="34" customWidth="1"/>
-    <col min="8" max="8" width="8.7109375" style="84" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" style="43" customWidth="1"/>
-    <col min="10" max="10" width="7.28515625" style="91" customWidth="1"/>
-    <col min="11" max="11" width="7.28515625" style="92" customWidth="1"/>
-    <col min="12" max="12" width="7.28515625" style="41" customWidth="1"/>
-    <col min="13" max="14" width="7.28515625" style="92" customWidth="1"/>
-    <col min="15" max="15" width="7.28515625" style="41" customWidth="1"/>
-    <col min="16" max="17" width="7.28515625" style="92" customWidth="1"/>
-    <col min="18" max="18" width="7.28515625" style="41" customWidth="1"/>
-    <col min="19" max="23" width="7.28515625" style="32" customWidth="1"/>
-    <col min="24" max="16384" width="9.140625" style="32"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:23" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="145" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="139" t="s">
-        <v>69</v>
-      </c>
-      <c r="D1" s="170" t="s">
-        <v>68</v>
-      </c>
-      <c r="E1" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" s="137" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" s="134" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="130" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" s="135" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" s="137" t="s">
-        <v>2</v>
-      </c>
-      <c r="K1" s="134"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="137" t="s">
-        <v>4</v>
-      </c>
-      <c r="N1" s="134"/>
-      <c r="O1" s="138"/>
-      <c r="P1" s="137" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q1" s="134"/>
-      <c r="R1" s="138"/>
-    </row>
-    <row r="2" spans="1:23" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128"/>
-      <c r="B2" s="146"/>
-      <c r="C2" s="140"/>
-      <c r="D2" s="124"/>
-      <c r="F2" s="141"/>
-      <c r="G2" s="129"/>
-      <c r="H2" s="131"/>
-      <c r="I2" s="136"/>
-      <c r="J2" s="111" t="s">
-        <v>36</v>
-      </c>
-      <c r="K2" s="110" t="s">
-        <v>37</v>
-      </c>
-      <c r="L2" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="M2" s="110" t="s">
-        <v>36</v>
-      </c>
-      <c r="N2" s="110" t="s">
-        <v>37</v>
-      </c>
-      <c r="O2" s="52" t="s">
-        <v>50</v>
-      </c>
-      <c r="P2" s="110" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q2" s="110" t="s">
-        <v>37</v>
-      </c>
-      <c r="R2" s="52" t="s">
-        <v>51</v>
-      </c>
-      <c r="T2" s="129"/>
-      <c r="U2" s="129"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-    </row>
-    <row r="3" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="30">
-        <v>1064</v>
-      </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="45" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="37"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="84">
-        <v>157.86000000000001</v>
-      </c>
-      <c r="I3" s="83">
-        <f>H3</f>
-        <v>157.86000000000001</v>
-      </c>
-      <c r="J3" s="95">
-        <v>0.93100000000000005</v>
-      </c>
-      <c r="K3" s="96">
-        <v>0.374</v>
-      </c>
-      <c r="L3" s="90">
-        <f t="shared" ref="L3:L9" si="0">J3-K3</f>
-        <v>0.55700000000000005</v>
-      </c>
-      <c r="M3" s="96">
-        <v>0</v>
-      </c>
-      <c r="N3" s="96">
-        <v>1.2999999999999999E-2</v>
-      </c>
-      <c r="O3" s="90">
-        <f t="shared" ref="O3:O9" si="1">M3-N3</f>
-        <v>-1.2999999999999999E-2</v>
-      </c>
-      <c r="P3" s="96">
-        <v>6.9000000000000006E-2</v>
-      </c>
-      <c r="Q3" s="96">
-        <v>0.61299999999999999</v>
-      </c>
-      <c r="R3" s="90">
-        <f t="shared" ref="R3:R7" si="2">P3-Q3</f>
-        <v>-0.54400000000000004</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="C4" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="F4" s="44">
-        <v>115.17</v>
-      </c>
-      <c r="H4" s="84">
-        <v>78.930000000000007</v>
-      </c>
-      <c r="I4" s="43">
-        <f>F4+H4</f>
-        <v>194.10000000000002</v>
-      </c>
-      <c r="J4" s="91">
-        <v>0.93300000000000005</v>
-      </c>
-      <c r="K4" s="92">
-        <v>0.77100000000000002</v>
-      </c>
-      <c r="L4" s="90">
-        <f t="shared" si="0"/>
-        <v>0.16200000000000003</v>
-      </c>
-      <c r="M4" s="92">
-        <v>0</v>
-      </c>
-      <c r="N4" s="92">
-        <v>0.01</v>
-      </c>
-      <c r="O4" s="90">
-        <f t="shared" si="1"/>
-        <v>-0.01</v>
-      </c>
-      <c r="P4" s="92">
-        <v>6.7000000000000004E-2</v>
-      </c>
-      <c r="Q4" s="92">
-        <v>0.219</v>
-      </c>
-      <c r="R4" s="90">
-        <f t="shared" si="2"/>
-        <v>-0.152</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B5" s="71" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="F5" s="44">
-        <v>32.799999999999997</v>
-      </c>
-      <c r="H5" s="84">
-        <v>162</v>
-      </c>
-      <c r="I5" s="43">
-        <f>F5+H5</f>
-        <v>194.8</v>
-      </c>
-      <c r="J5" s="91">
-        <v>0.96399999999999997</v>
-      </c>
-      <c r="K5" s="92">
-        <v>0.83</v>
-      </c>
-      <c r="L5" s="90">
-        <f t="shared" si="0"/>
-        <v>0.13400000000000001</v>
-      </c>
-      <c r="M5" s="92">
-        <v>0</v>
-      </c>
-      <c r="N5" s="92">
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="O5" s="90">
-        <f t="shared" si="1"/>
-        <v>-8.0000000000000002E-3</v>
-      </c>
-      <c r="P5" s="92">
-        <v>3.5999999999999997E-2</v>
-      </c>
-      <c r="Q5" s="92">
-        <v>0.16200000000000001</v>
-      </c>
-      <c r="R5" s="90">
-        <f t="shared" si="2"/>
-        <v>-0.126</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B6" s="71" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="F6" s="172">
-        <v>68.25</v>
-      </c>
-      <c r="H6" s="84">
-        <v>125</v>
-      </c>
-      <c r="I6" s="43">
-        <f>F6+H6</f>
-        <v>193.25</v>
-      </c>
-      <c r="J6" s="91">
-        <v>0.96399999999999997</v>
-      </c>
-      <c r="K6" s="92">
-        <v>0.70099999999999996</v>
-      </c>
-      <c r="L6" s="90">
-        <f t="shared" si="0"/>
-        <v>0.26300000000000001</v>
-      </c>
-      <c r="M6" s="92">
-        <v>0</v>
-      </c>
-      <c r="N6" s="92">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="O6" s="90">
-        <f t="shared" si="1"/>
-        <v>-1.7999999999999999E-2</v>
-      </c>
-      <c r="P6" s="92">
-        <v>3.5999999999999997E-2</v>
-      </c>
-      <c r="Q6" s="92">
-        <v>0.28100000000000003</v>
-      </c>
-      <c r="R6" s="90">
-        <f t="shared" si="2"/>
-        <v>-0.24500000000000002</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="C7" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="F7" s="44">
-        <v>136.35</v>
-      </c>
-      <c r="G7" s="34">
-        <v>115.17</v>
-      </c>
-      <c r="H7" s="84">
-        <v>78.930000000000007</v>
-      </c>
-      <c r="I7" s="43">
-        <f>SUM(F7:H7)</f>
-        <v>330.45</v>
-      </c>
-      <c r="J7" s="91">
-        <v>0.93300000000000005</v>
-      </c>
-      <c r="K7" s="92">
-        <v>0.77100000000000002</v>
-      </c>
-      <c r="L7" s="90">
-        <f t="shared" si="0"/>
-        <v>0.16200000000000003</v>
-      </c>
-      <c r="M7" s="92">
-        <v>0</v>
-      </c>
-      <c r="N7" s="92">
-        <v>0.01</v>
-      </c>
-      <c r="O7" s="90">
-        <f t="shared" si="1"/>
-        <v>-0.01</v>
-      </c>
-      <c r="P7" s="92">
-        <v>6.7000000000000004E-2</v>
-      </c>
-      <c r="Q7" s="92">
-        <v>0.218</v>
-      </c>
-      <c r="R7" s="90">
-        <f t="shared" si="2"/>
-        <v>-0.151</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" s="30"/>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" s="30"/>
-      <c r="D10" s="37"/>
-      <c r="L10" s="97"/>
-      <c r="O10" s="97"/>
-      <c r="R10" s="97"/>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B11" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" s="38" t="s">
-        <v>103</v>
-      </c>
-      <c r="F11" s="44">
-        <v>181.31</v>
-      </c>
-      <c r="G11" s="34">
-        <v>193.08</v>
-      </c>
-      <c r="H11" s="84">
-        <v>157.86000000000001</v>
-      </c>
-      <c r="I11" s="43">
-        <f>SUM(F11:H11)</f>
-        <v>532.25</v>
-      </c>
-      <c r="J11" s="91">
-        <v>0.94899999999999995</v>
-      </c>
-      <c r="K11" s="92">
-        <v>0.56100000000000005</v>
-      </c>
-      <c r="L11" s="90">
-        <f>J11-K11</f>
-        <v>0.3879999999999999</v>
-      </c>
-      <c r="M11" s="92">
-        <v>0</v>
-      </c>
-      <c r="N11" s="92">
-        <v>1.9E-2</v>
-      </c>
-      <c r="O11" s="90">
-        <f>M11-N11</f>
-        <v>-1.9E-2</v>
-      </c>
-      <c r="P11" s="92">
-        <v>5.0999999999999997E-2</v>
-      </c>
-      <c r="Q11" s="92">
-        <v>0.42</v>
-      </c>
-      <c r="R11" s="90">
-        <f>P11-Q11</f>
-        <v>-0.36899999999999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B12" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C12" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="F12" s="44">
-        <v>164.55</v>
-      </c>
-      <c r="G12" s="34">
-        <v>193.08</v>
-      </c>
-      <c r="H12" s="84">
-        <v>157.86000000000001</v>
-      </c>
-      <c r="I12" s="43">
-        <f>SUM(F12:H12)</f>
-        <v>515.49</v>
-      </c>
-      <c r="J12" s="91">
-        <v>0.96299999999999997</v>
-      </c>
-      <c r="K12" s="92">
-        <v>0.623</v>
-      </c>
-      <c r="L12" s="90">
-        <f>J12-K12</f>
-        <v>0.33999999999999997</v>
-      </c>
-      <c r="M12" s="92">
-        <v>0</v>
-      </c>
-      <c r="N12" s="92">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="O12" s="90">
-        <f>M12-N12</f>
-        <v>-1.7999999999999999E-2</v>
-      </c>
-      <c r="P12" s="92">
-        <v>3.6999999999999998E-2</v>
-      </c>
-      <c r="Q12" s="92">
-        <v>0.35899999999999999</v>
-      </c>
-      <c r="R12" s="90">
-        <f>P12-Q12</f>
-        <v>-0.32200000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B13" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C13" s="38" t="s">
-        <v>101</v>
-      </c>
-      <c r="D13" s="37"/>
-      <c r="F13" s="44">
-        <v>133.22999999999999</v>
-      </c>
-      <c r="G13" s="34">
-        <v>164.55</v>
-      </c>
-      <c r="H13" s="84">
-        <v>157.86000000000001</v>
-      </c>
-      <c r="I13" s="43">
-        <f>SUM(F13:H13)</f>
-        <v>455.64</v>
-      </c>
-      <c r="J13" s="91">
-        <v>0.96399999999999997</v>
-      </c>
-      <c r="K13" s="92">
-        <v>0.82899999999999996</v>
-      </c>
-      <c r="L13" s="90">
-        <f>J13-K13</f>
-        <v>0.13500000000000001</v>
-      </c>
-      <c r="M13" s="92">
-        <v>0</v>
-      </c>
-      <c r="N13" s="92">
-        <v>1.9E-2</v>
-      </c>
-      <c r="O13" s="90">
-        <f>M13-N13</f>
-        <v>-1.9E-2</v>
-      </c>
-      <c r="P13" s="92">
-        <v>3.5999999999999997E-2</v>
-      </c>
-      <c r="Q13" s="92">
-        <v>0.152</v>
-      </c>
-      <c r="R13" s="90">
-        <f>P13-Q13</f>
-        <v>-0.11599999999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B14" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="F14" s="44">
-        <v>115.17</v>
-      </c>
-      <c r="G14" s="34">
-        <v>133.22999999999999</v>
-      </c>
-      <c r="H14" s="84">
-        <v>157.86000000000001</v>
-      </c>
-      <c r="I14" s="43">
-        <f>SUM(F14:H14)</f>
-        <v>406.26</v>
-      </c>
-      <c r="J14" s="91">
-        <v>0.96199999999999997</v>
-      </c>
-      <c r="K14" s="92">
-        <v>0.93799999999999994</v>
-      </c>
-      <c r="L14" s="90">
-        <f>J14-K14</f>
-        <v>2.4000000000000021E-2</v>
-      </c>
-      <c r="M14" s="92">
-        <v>0</v>
-      </c>
-      <c r="N14" s="92">
-        <v>1.9E-2</v>
-      </c>
-      <c r="O14" s="90">
-        <f>M14-N14</f>
-        <v>-1.9E-2</v>
-      </c>
-      <c r="P14" s="92">
-        <v>3.7999999999999999E-2</v>
-      </c>
-      <c r="Q14" s="92">
-        <v>4.2999999999999997E-2</v>
-      </c>
-      <c r="R14" s="90">
-        <f>P14-Q14</f>
-        <v>-4.9999999999999975E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="71"/>
-      <c r="L18" s="97"/>
-      <c r="O18" s="97"/>
-      <c r="R18" s="97"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="71"/>
-      <c r="L19" s="97"/>
-      <c r="O19" s="97"/>
-      <c r="R19" s="97"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="L20" s="97"/>
-      <c r="O20" s="97"/>
-      <c r="R20" s="97"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="L21" s="97"/>
-      <c r="O21" s="97"/>
-      <c r="R21" s="97"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="C23" s="37"/>
-      <c r="F23" s="122"/>
-      <c r="L23" s="97"/>
-      <c r="O23" s="97"/>
-      <c r="R23" s="97"/>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="30"/>
-      <c r="F24" s="122"/>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="F25" s="122"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="30"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="30"/>
-      <c r="C27" s="118"/>
-      <c r="D27" s="171"/>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="30"/>
-    </row>
-  </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="B1:B2"/>
-  </mergeCells>
-  <conditionalFormatting sqref="L10:L17">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
-      <formula>$L$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L16:L17">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
-      <formula>0.45</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="greaterThan">
-      <formula>0.45</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L18:L21">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L23">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
-      <formula>$L$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03EBE129-7102-4E9D-8A3D-9B26EFEE1948}">
   <dimension ref="A1:Y21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10807,63 +12050,63 @@
       <c r="A1" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="127" t="s">
+      <c r="B1" s="133" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="152" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="139" t="s">
+      <c r="D1" s="135" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="137" t="s">
+      <c r="E1" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="134" t="s">
+      <c r="F1" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="142" t="s">
+      <c r="G1" s="144" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="142" t="s">
+      <c r="H1" s="144" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="134" t="s">
+      <c r="I1" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="135" t="s">
+      <c r="J1" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="137" t="s">
+      <c r="K1" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="134"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="137" t="s">
+      <c r="L1" s="131"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="134"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="137" t="s">
+      <c r="O1" s="131"/>
+      <c r="P1" s="132"/>
+      <c r="Q1" s="130" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="134"/>
-      <c r="S1" s="138"/>
+      <c r="R1" s="131"/>
+      <c r="S1" s="132"/>
       <c r="T1" s="153" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="129"/>
-      <c r="B2" s="128"/>
-      <c r="C2" s="144"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="129"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="136"/>
+      <c r="A2" s="127"/>
+      <c r="B2" s="134"/>
+      <c r="C2" s="146"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="134"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="129"/>
       <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
@@ -10892,10 +12135,10 @@
         <v>51</v>
       </c>
       <c r="T2" s="154"/>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
     </row>
     <row r="3" spans="1:25" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="30">
@@ -11786,7 +13029,7 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="M9:M19">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>0.45</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan">
@@ -11794,386 +13037,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M9:M20">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>$M$8</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BF2213B-BB65-498C-AA64-42693820505C}">
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" style="17" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" style="17" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" style="17" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="17" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="17"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="169" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="169" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="164" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="164" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="164" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="165" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="165"/>
-      <c r="H1" s="158" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="158"/>
-      <c r="J1" s="159" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="159"/>
-    </row>
-    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="169"/>
-      <c r="B2" s="169"/>
-      <c r="C2" s="164"/>
-      <c r="D2" s="164"/>
-      <c r="E2" s="164"/>
-      <c r="F2" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="160" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="160">
-        <v>1550</v>
-      </c>
-      <c r="D3" s="160" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="13">
-        <v>52</v>
-      </c>
-      <c r="F3" s="14">
-        <v>0.48</v>
-      </c>
-      <c r="G3" s="14">
-        <v>0.16</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="K3" s="16" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="161"/>
-      <c r="B4" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="161"/>
-      <c r="D4" s="163"/>
-      <c r="E4" s="18">
-        <v>52</v>
-      </c>
-      <c r="F4" s="27">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="G4" s="27">
-        <v>0.11</v>
-      </c>
-      <c r="H4" s="28">
-        <v>0.44</v>
-      </c>
-      <c r="I4" s="28">
-        <v>0.38</v>
-      </c>
-      <c r="J4" s="29">
-        <v>0</v>
-      </c>
-      <c r="K4" s="29">
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="161"/>
-      <c r="B5" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="161"/>
-      <c r="D5" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="19">
-        <f>2.6*2</f>
-        <v>5.2</v>
-      </c>
-      <c r="F5" s="20">
-        <v>0.41</v>
-      </c>
-      <c r="G5" s="20">
-        <v>0.04</v>
-      </c>
-      <c r="H5" s="21">
-        <v>0.59</v>
-      </c>
-      <c r="I5" s="21">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="J5" s="22">
-        <v>0</v>
-      </c>
-      <c r="K5" s="22">
-        <v>0.67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="162"/>
-      <c r="B6" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="162"/>
-      <c r="D6" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="23">
-        <f>6.6*2</f>
-        <v>13.2</v>
-      </c>
-      <c r="F6" s="24">
-        <v>0.41</v>
-      </c>
-      <c r="G6" s="24">
-        <v>0.04</v>
-      </c>
-      <c r="H6" s="25">
-        <v>0.59</v>
-      </c>
-      <c r="I6" s="25">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="J6" s="26">
-        <v>0</v>
-      </c>
-      <c r="K6" s="26">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="166" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="166">
-        <v>1320</v>
-      </c>
-      <c r="D7" s="166" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="3">
-        <v>100</v>
-      </c>
-      <c r="F7" s="10">
-        <v>0.23</v>
-      </c>
-      <c r="G7" s="10">
-        <v>0.05</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J7" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="K7" s="12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="167"/>
-      <c r="B8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="167"/>
-      <c r="D8" s="168"/>
-      <c r="E8" s="1">
-        <v>100</v>
-      </c>
-      <c r="F8" s="7">
-        <v>0.17</v>
-      </c>
-      <c r="G8" s="7">
-        <v>0.02</v>
-      </c>
-      <c r="H8" s="8">
-        <v>0.15</v>
-      </c>
-      <c r="I8" s="8">
-        <v>0.19</v>
-      </c>
-      <c r="J8" s="9">
-        <v>0.67</v>
-      </c>
-      <c r="K8" s="9">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="167"/>
-      <c r="B9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="167"/>
-      <c r="D9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="2">
-        <f>3.5*2</f>
-        <v>7</v>
-      </c>
-      <c r="F9" s="4">
-        <v>0.41</v>
-      </c>
-      <c r="G9" s="4">
-        <v>0.08</v>
-      </c>
-      <c r="H9" s="5">
-        <v>0.59</v>
-      </c>
-      <c r="I9" s="5">
-        <v>0.4</v>
-      </c>
-      <c r="J9" s="6">
-        <v>0</v>
-      </c>
-      <c r="K9" s="6">
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="167"/>
-      <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="167"/>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="2">
-        <f>13.9*2</f>
-        <v>27.8</v>
-      </c>
-      <c r="F10" s="4">
-        <v>0.16</v>
-      </c>
-      <c r="G10" s="4">
-        <v>0.03</v>
-      </c>
-      <c r="H10" s="5">
-        <v>0.83</v>
-      </c>
-      <c r="I10" s="5">
-        <v>0.36</v>
-      </c>
-      <c r="J10" s="6">
-        <v>0</v>
-      </c>
-      <c r="K10" s="6">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="168"/>
-      <c r="B11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="168"/>
-      <c r="D11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="2">
-        <f>8.5*2</f>
-        <v>17</v>
-      </c>
-      <c r="F11" s="4">
-        <v>0.38</v>
-      </c>
-      <c r="G11" s="4">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="H11" s="5">
-        <v>0.62</v>
-      </c>
-      <c r="I11" s="5">
-        <v>0.39</v>
-      </c>
-      <c r="J11" s="6">
-        <v>0</v>
-      </c>
-      <c r="K11" s="6">
-        <v>0.54</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>